<commit_message>
3rd release with additional data
- corrections on previous data to delete redundancies
- L2 corrector data added
</commit_message>
<xml_diff>
--- a/006_DASSAULT_AETHER/gridConvergence_D01_V1.xlsx
+++ b/006_DASSAULT_AETHER/gridConvergence_D01_V1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\DA\SOC\NP\ORG\DGT\UNIX\SCIENTIFIQUE\CSC\PROJET\GIVRE\IPW3\006_DASSAULT_AETHER\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91B77E6E-D3AA-49B3-967C-A1549BF5FDD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D919AF0A-BA65-45A4-8D86-F3380B61E778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INSTRUCTIONS" sheetId="1" r:id="rId1"/>
@@ -538,7 +538,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -670,11 +670,22 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -808,6 +819,7 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -832,7 +844,13 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -844,13 +862,7 @@
     <xf numFmtId="165" fontId="5" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -862,6 +874,12 @@
     <xf numFmtId="165" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -871,16 +889,10 @@
     <xf numFmtId="165" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1284,341 +1296,341 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E78"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="18"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="17.5"/>
   <cols>
-    <col min="1" max="1" width="96.33203125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" customWidth="1"/>
-    <col min="5" max="5" width="16.33203125" customWidth="1"/>
-    <col min="6" max="6" width="17.44140625" customWidth="1"/>
-    <col min="7" max="7" width="14.44140625" customWidth="1"/>
+    <col min="1" max="1" width="96.3046875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="20.765625" customWidth="1"/>
+    <col min="5" max="5" width="16.3046875" customWidth="1"/>
+    <col min="6" max="6" width="17.4609375" customWidth="1"/>
+    <col min="7" max="7" width="14.4609375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="15">
-      <c r="A1" s="47" t="s">
+    <row r="1" spans="1:1" ht="15.5">
+      <c r="A1" s="48" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="15">
-      <c r="A2" s="47"/>
-    </row>
-    <row r="3" spans="1:1" ht="15">
-      <c r="A3" s="47"/>
-    </row>
-    <row r="4" spans="1:1" ht="15">
-      <c r="A4" s="47" t="s">
+    <row r="2" spans="1:1" ht="15.5">
+      <c r="A2" s="48"/>
+    </row>
+    <row r="3" spans="1:1" ht="15.5">
+      <c r="A3" s="48"/>
+    </row>
+    <row r="4" spans="1:1" ht="15.5">
+      <c r="A4" s="48" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="15">
-      <c r="A5" s="47"/>
-    </row>
-    <row r="6" spans="1:1" ht="20.25">
+    <row r="5" spans="1:1" ht="15.5">
+      <c r="A5" s="48"/>
+    </row>
+    <row r="6" spans="1:1" ht="20">
       <c r="A6" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="20.25">
+    <row r="7" spans="1:1" ht="20">
       <c r="A7" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="20.25">
+    <row r="8" spans="1:1" ht="20">
       <c r="A8" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="20.25">
+    <row r="9" spans="1:1" ht="20">
       <c r="A9" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="20.25">
+    <row r="10" spans="1:1" ht="20">
       <c r="A10" s="3" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="20.25">
+    <row r="11" spans="1:1" ht="20">
       <c r="A11" s="3" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="12" spans="1:1" ht="20.25">
+    <row r="12" spans="1:1" ht="20">
       <c r="A12" s="3" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="1:1" ht="15">
-      <c r="A13" s="48" t="s">
+    <row r="13" spans="1:1" ht="15.5">
+      <c r="A13" s="49" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="15">
-      <c r="A14" s="48"/>
-    </row>
-    <row r="15" spans="1:1" ht="20.25">
+    <row r="14" spans="1:1" ht="15.5">
+      <c r="A14" s="49"/>
+    </row>
+    <row r="15" spans="1:1" ht="20">
       <c r="A15" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:1" ht="20.25">
+    <row r="16" spans="1:1" ht="20">
       <c r="A16" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="20.25">
+    <row r="17" spans="1:5" ht="20">
       <c r="A17" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="20.25">
+    <row r="18" spans="1:5" ht="20">
       <c r="A18" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="20.25">
+    <row r="19" spans="1:5" ht="20">
       <c r="A19" s="3" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="15">
-      <c r="A20" s="47" t="s">
+    <row r="20" spans="1:5" ht="15.5">
+      <c r="A20" s="48" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="15">
-      <c r="A21" s="47"/>
-    </row>
-    <row r="22" spans="1:5" ht="20.25">
+    <row r="21" spans="1:5" ht="15.5">
+      <c r="A21" s="48"/>
+    </row>
+    <row r="22" spans="1:5" ht="20">
       <c r="A22" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="20.25">
+    <row r="23" spans="1:5" ht="20">
       <c r="A23" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="20.25">
+    <row r="24" spans="1:5" ht="20">
       <c r="A24" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="20.25">
+    <row r="25" spans="1:5" ht="20">
       <c r="A25" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="20.25">
+    <row r="26" spans="1:5" ht="20">
       <c r="A26" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="20.25">
+    <row r="27" spans="1:5" ht="20">
       <c r="A27" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E27" s="4"/>
     </row>
-    <row r="28" spans="1:5" ht="20.25">
+    <row r="28" spans="1:5" ht="20">
       <c r="A28" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="20.25">
+    <row r="29" spans="1:5" ht="20">
       <c r="A29" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="20.25">
+    <row r="30" spans="1:5" ht="20">
       <c r="A30" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E30" s="4"/>
     </row>
-    <row r="31" spans="1:5" ht="20.25">
+    <row r="31" spans="1:5" ht="20">
       <c r="A31" s="3" t="s">
         <v>21</v>
       </c>
       <c r="E31" s="4"/>
     </row>
-    <row r="32" spans="1:5" ht="15">
-      <c r="A32" s="47" t="s">
+    <row r="32" spans="1:5" ht="15.5">
+      <c r="A32" s="48" t="s">
         <v>22</v>
       </c>
       <c r="E32" s="4"/>
     </row>
-    <row r="33" spans="1:5" ht="15">
-      <c r="A33" s="47"/>
+    <row r="33" spans="1:5" ht="15.5">
+      <c r="A33" s="48"/>
       <c r="E33" s="4"/>
     </row>
-    <row r="34" spans="1:5" ht="20.25">
+    <row r="34" spans="1:5" ht="20">
       <c r="A34" s="3" t="s">
         <v>12</v>
       </c>
       <c r="E34" s="4"/>
     </row>
-    <row r="35" spans="1:5" ht="20.25">
+    <row r="35" spans="1:5" ht="20">
       <c r="A35" s="3" t="s">
         <v>13</v>
       </c>
       <c r="E35" s="4"/>
     </row>
-    <row r="36" spans="1:5" ht="20.25">
+    <row r="36" spans="1:5" ht="20">
       <c r="A36" s="3" t="s">
         <v>14</v>
       </c>
       <c r="E36" s="4"/>
     </row>
-    <row r="37" spans="1:5" ht="20.25">
+    <row r="37" spans="1:5" ht="20">
       <c r="A37" s="3" t="s">
         <v>23</v>
       </c>
       <c r="E37" s="4"/>
     </row>
-    <row r="38" spans="1:5" ht="20.25">
+    <row r="38" spans="1:5" ht="20">
       <c r="A38" s="3" t="s">
         <v>24</v>
       </c>
       <c r="E38" s="4"/>
     </row>
-    <row r="39" spans="1:5" ht="20.25">
+    <row r="39" spans="1:5" ht="20">
       <c r="A39" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="20.25">
+    <row r="40" spans="1:5" ht="20">
       <c r="A40" s="3" t="s">
         <v>18</v>
       </c>
       <c r="E40" s="4"/>
     </row>
-    <row r="41" spans="1:5" ht="20.25">
+    <row r="41" spans="1:5" ht="20">
       <c r="A41" s="3" t="s">
         <v>19</v>
       </c>
       <c r="E41" s="4"/>
     </row>
-    <row r="42" spans="1:5" ht="20.25">
+    <row r="42" spans="1:5" ht="20">
       <c r="A42" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E42" s="4"/>
     </row>
-    <row r="43" spans="1:5" ht="20.25">
+    <row r="43" spans="1:5" ht="20">
       <c r="A43" s="3" t="s">
         <v>21</v>
       </c>
       <c r="E43" s="4"/>
     </row>
-    <row r="44" spans="1:5" ht="15">
-      <c r="A44" s="47" t="s">
+    <row r="44" spans="1:5" ht="15.5">
+      <c r="A44" s="48" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="45" spans="1:5" ht="15">
-      <c r="A45" s="47"/>
+    <row r="45" spans="1:5" ht="15.5">
+      <c r="A45" s="48"/>
       <c r="E45" s="4"/>
     </row>
-    <row r="46" spans="1:5" ht="20.25">
+    <row r="46" spans="1:5" ht="20">
       <c r="A46" s="3" t="s">
         <v>26</v>
       </c>
       <c r="E46" s="4"/>
     </row>
-    <row r="47" spans="1:5" ht="20.25">
+    <row r="47" spans="1:5" ht="20">
       <c r="A47" s="3" t="s">
         <v>27</v>
       </c>
       <c r="E47" s="4"/>
     </row>
-    <row r="48" spans="1:5" ht="20.25">
+    <row r="48" spans="1:5" ht="20">
       <c r="A48" s="3" t="s">
         <v>28</v>
       </c>
       <c r="E48" s="4"/>
     </row>
-    <row r="49" spans="1:5" ht="20.25">
+    <row r="49" spans="1:5" ht="20">
       <c r="A49" s="3" t="s">
         <v>29</v>
       </c>
       <c r="E49" s="4"/>
     </row>
-    <row r="50" spans="1:5" ht="20.25">
+    <row r="50" spans="1:5" ht="20">
       <c r="A50" s="3" t="s">
         <v>30</v>
       </c>
       <c r="E50" s="4"/>
     </row>
-    <row r="51" spans="1:5" ht="20.25">
+    <row r="51" spans="1:5" ht="20">
       <c r="A51" s="3" t="s">
         <v>31</v>
       </c>
       <c r="E51" s="4"/>
     </row>
-    <row r="52" spans="1:5" ht="20.25">
+    <row r="52" spans="1:5" ht="20">
       <c r="A52" s="3" t="s">
         <v>32</v>
       </c>
       <c r="E52" s="4"/>
     </row>
-    <row r="53" spans="1:5" ht="20.25">
+    <row r="53" spans="1:5" ht="20">
       <c r="A53" s="3" t="s">
         <v>33</v>
       </c>
       <c r="E53" s="4"/>
     </row>
-    <row r="54" spans="1:5" ht="20.25">
+    <row r="54" spans="1:5" ht="20">
       <c r="A54" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E54" s="4"/>
     </row>
-    <row r="55" spans="1:5" ht="20.25">
+    <row r="55" spans="1:5" ht="20">
       <c r="A55" s="3" t="s">
         <v>34</v>
       </c>
       <c r="E55" s="4"/>
     </row>
-    <row r="56" spans="1:5" ht="15">
-      <c r="A56" s="47" t="s">
+    <row r="56" spans="1:5" ht="15.5">
+      <c r="A56" s="48" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="57" spans="1:5" ht="15">
-      <c r="A57" s="47"/>
+    <row r="57" spans="1:5" ht="15.5">
+      <c r="A57" s="48"/>
       <c r="E57" s="4"/>
     </row>
-    <row r="58" spans="1:5" ht="20.25">
+    <row r="58" spans="1:5" ht="20">
       <c r="A58" s="1" t="s">
         <v>36</v>
       </c>
       <c r="E58" s="4"/>
     </row>
-    <row r="59" spans="1:5" ht="20.25">
+    <row r="59" spans="1:5" ht="20">
       <c r="A59" s="5" t="s">
         <v>37</v>
       </c>
       <c r="E59" s="4"/>
     </row>
-    <row r="60" spans="1:5" ht="20.25">
+    <row r="60" spans="1:5" ht="20">
       <c r="A60" s="3" t="s">
         <v>68</v>
       </c>
       <c r="E60" s="4"/>
     </row>
-    <row r="61" spans="1:5" ht="20.25">
+    <row r="61" spans="1:5" ht="20">
       <c r="A61" s="1" t="s">
         <v>38</v>
       </c>
       <c r="E61" s="4"/>
     </row>
-    <row r="62" spans="1:5" ht="20.25">
+    <row r="62" spans="1:5" ht="20">
       <c r="A62" s="3" t="s">
         <v>37</v>
       </c>
       <c r="E62" s="4"/>
     </row>
-    <row r="63" spans="1:5" ht="20.25">
+    <row r="63" spans="1:5" ht="20">
       <c r="A63" s="3" t="s">
         <v>39</v>
       </c>
@@ -1684,36 +1696,36 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:AMG78"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.77734375" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.765625" defaultRowHeight="15.5"/>
   <cols>
-    <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.69140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.07421875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.44140625" style="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.109375" style="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.4609375" style="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.07421875" style="10" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13" style="10" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="31.44140625" style="10" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="24.109375" style="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31.4609375" style="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.07421875" style="10" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13" style="10" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="31.44140625" style="10" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="24.109375" style="10" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="31.4609375" style="10" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="24.07421875" style="10" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="13" style="10" bestFit="1" customWidth="1"/>
-    <col min="13" max="18" width="13.6640625" style="10" customWidth="1"/>
-    <col min="19" max="1021" width="10.77734375" style="10"/>
+    <col min="13" max="18" width="13.69140625" style="10" customWidth="1"/>
+    <col min="19" max="1021" width="10.765625" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1021" s="32" customFormat="1" ht="25.5">
-      <c r="D1" s="51" t="s">
+    <row r="1" spans="1:1021" s="32" customFormat="1" ht="25">
+      <c r="D1" s="52" t="s">
         <v>44</v>
       </c>
-      <c r="E1" s="51"/>
-      <c r="F1" s="51"/>
-      <c r="G1" s="51"/>
-      <c r="H1" s="51"/>
-      <c r="I1" s="51"/>
-      <c r="J1" s="51"/>
-      <c r="K1" s="51"/>
-      <c r="L1" s="51"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="52"/>
+      <c r="H1" s="52"/>
+      <c r="I1" s="52"/>
+      <c r="J1" s="52"/>
+      <c r="K1" s="52"/>
+      <c r="L1" s="52"/>
       <c r="M1" s="31"/>
       <c r="N1" s="31"/>
       <c r="O1" s="31"/>
@@ -2724,37 +2736,37 @@
       <c r="AMF1" s="31"/>
       <c r="AMG1" s="31"/>
     </row>
-    <row r="2" spans="1:1021" s="6" customFormat="1" ht="59.1" customHeight="1">
-      <c r="A2" s="65" t="s">
+    <row r="2" spans="1:1021" s="6" customFormat="1" ht="59.15" customHeight="1">
+      <c r="A2" s="68" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="66"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="66"/>
-      <c r="G2" s="66"/>
-      <c r="H2" s="66"/>
-      <c r="I2" s="66"/>
-      <c r="J2" s="66"/>
-      <c r="K2" s="66"/>
-      <c r="L2" s="67"/>
-    </row>
-    <row r="3" spans="1:1021" s="32" customFormat="1" ht="25.5">
-      <c r="A3" s="62" t="s">
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="70"/>
+    </row>
+    <row r="3" spans="1:1021" s="32" customFormat="1" ht="25">
+      <c r="A3" s="63" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="63"/>
-      <c r="D3" s="63"/>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
-      <c r="G3" s="63"/>
-      <c r="H3" s="63"/>
-      <c r="I3" s="63"/>
-      <c r="J3" s="63"/>
-      <c r="K3" s="63"/>
-      <c r="L3" s="64"/>
+      <c r="B3" s="64"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="64"/>
+      <c r="H3" s="64"/>
+      <c r="I3" s="64"/>
+      <c r="J3" s="64"/>
+      <c r="K3" s="64"/>
+      <c r="L3" s="65"/>
       <c r="M3" s="31"/>
       <c r="N3" s="31"/>
       <c r="O3" s="31"/>
@@ -3765,27 +3777,27 @@
       <c r="AMF3" s="31"/>
       <c r="AMG3" s="31"/>
     </row>
-    <row r="4" spans="1:1021" s="32" customFormat="1" ht="25.5">
-      <c r="A4" s="56" t="s">
+    <row r="4" spans="1:1021" s="32" customFormat="1" ht="25">
+      <c r="A4" s="59" t="s">
         <v>60</v>
       </c>
-      <c r="B4" s="57"/>
-      <c r="C4" s="58"/>
-      <c r="D4" s="55" t="s">
+      <c r="B4" s="60"/>
+      <c r="C4" s="61"/>
+      <c r="D4" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="E4" s="55"/>
-      <c r="F4" s="55"/>
-      <c r="G4" s="55" t="s">
+      <c r="E4" s="62"/>
+      <c r="F4" s="62"/>
+      <c r="G4" s="62" t="s">
         <v>48</v>
       </c>
-      <c r="H4" s="55"/>
-      <c r="I4" s="55"/>
-      <c r="J4" s="55" t="s">
+      <c r="H4" s="62"/>
+      <c r="I4" s="62"/>
+      <c r="J4" s="62" t="s">
         <v>49</v>
       </c>
-      <c r="K4" s="55"/>
-      <c r="L4" s="55"/>
+      <c r="K4" s="62"/>
+      <c r="L4" s="62"/>
       <c r="M4" s="31"/>
       <c r="N4" s="31"/>
       <c r="O4" s="21"/>
@@ -5059,21 +5071,21 @@
       <c r="M21" s="15"/>
       <c r="N21" s="15"/>
     </row>
-    <row r="22" spans="1:1021" s="32" customFormat="1" ht="25.5">
-      <c r="A22" s="55" t="s">
+    <row r="22" spans="1:1021" s="32" customFormat="1" ht="25">
+      <c r="A22" s="62" t="s">
         <v>57</v>
       </c>
-      <c r="B22" s="55"/>
-      <c r="C22" s="55"/>
-      <c r="D22" s="55"/>
-      <c r="E22" s="55"/>
-      <c r="F22" s="55"/>
-      <c r="G22" s="55"/>
-      <c r="H22" s="55"/>
-      <c r="I22" s="55"/>
-      <c r="J22" s="55"/>
-      <c r="K22" s="55"/>
-      <c r="L22" s="55"/>
+      <c r="B22" s="62"/>
+      <c r="C22" s="62"/>
+      <c r="D22" s="62"/>
+      <c r="E22" s="62"/>
+      <c r="F22" s="62"/>
+      <c r="G22" s="62"/>
+      <c r="H22" s="62"/>
+      <c r="I22" s="62"/>
+      <c r="J22" s="62"/>
+      <c r="K22" s="62"/>
+      <c r="L22" s="62"/>
       <c r="M22" s="33"/>
       <c r="N22" s="33"/>
       <c r="O22" s="31"/>
@@ -6084,27 +6096,27 @@
       <c r="AMF22" s="31"/>
       <c r="AMG22" s="31"/>
     </row>
-    <row r="23" spans="1:1021" s="32" customFormat="1" ht="25.5">
-      <c r="A23" s="56" t="s">
+    <row r="23" spans="1:1021" s="32" customFormat="1" ht="25">
+      <c r="A23" s="59" t="s">
         <v>60</v>
       </c>
-      <c r="B23" s="57"/>
-      <c r="C23" s="58"/>
-      <c r="D23" s="55" t="s">
+      <c r="B23" s="60"/>
+      <c r="C23" s="61"/>
+      <c r="D23" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="E23" s="55"/>
-      <c r="F23" s="55"/>
-      <c r="G23" s="55" t="s">
+      <c r="E23" s="62"/>
+      <c r="F23" s="62"/>
+      <c r="G23" s="62" t="s">
         <v>48</v>
       </c>
-      <c r="H23" s="55"/>
-      <c r="I23" s="55"/>
-      <c r="J23" s="55" t="s">
+      <c r="H23" s="62"/>
+      <c r="I23" s="62"/>
+      <c r="J23" s="62" t="s">
         <v>49</v>
       </c>
-      <c r="K23" s="55"/>
-      <c r="L23" s="55"/>
+      <c r="K23" s="62"/>
+      <c r="L23" s="62"/>
       <c r="M23" s="31"/>
       <c r="N23" s="31"/>
       <c r="O23" s="31"/>
@@ -7376,21 +7388,21 @@
       <c r="K40" s="44"/>
       <c r="L40" s="24"/>
     </row>
-    <row r="41" spans="1:1021" s="32" customFormat="1" ht="25.5">
-      <c r="A41" s="68" t="s">
+    <row r="41" spans="1:1021" s="32" customFormat="1" ht="25">
+      <c r="A41" s="67" t="s">
         <v>58</v>
       </c>
-      <c r="B41" s="68"/>
-      <c r="C41" s="68"/>
-      <c r="D41" s="68"/>
-      <c r="E41" s="68"/>
-      <c r="F41" s="68"/>
-      <c r="G41" s="68"/>
-      <c r="H41" s="68"/>
-      <c r="I41" s="68"/>
-      <c r="J41" s="68"/>
-      <c r="K41" s="68"/>
-      <c r="L41" s="68"/>
+      <c r="B41" s="67"/>
+      <c r="C41" s="67"/>
+      <c r="D41" s="67"/>
+      <c r="E41" s="67"/>
+      <c r="F41" s="67"/>
+      <c r="G41" s="67"/>
+      <c r="H41" s="67"/>
+      <c r="I41" s="67"/>
+      <c r="J41" s="67"/>
+      <c r="K41" s="67"/>
+      <c r="L41" s="67"/>
       <c r="M41" s="31"/>
       <c r="N41" s="31"/>
       <c r="O41" s="31"/>
@@ -8401,27 +8413,27 @@
       <c r="AMF41" s="31"/>
       <c r="AMG41" s="31"/>
     </row>
-    <row r="42" spans="1:1021" s="32" customFormat="1" ht="25.5">
-      <c r="A42" s="56" t="s">
+    <row r="42" spans="1:1021" s="32" customFormat="1" ht="25">
+      <c r="A42" s="59" t="s">
         <v>60</v>
       </c>
-      <c r="B42" s="57"/>
-      <c r="C42" s="58"/>
-      <c r="D42" s="55" t="s">
+      <c r="B42" s="60"/>
+      <c r="C42" s="61"/>
+      <c r="D42" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="E42" s="55"/>
-      <c r="F42" s="55"/>
-      <c r="G42" s="55" t="s">
+      <c r="E42" s="62"/>
+      <c r="F42" s="62"/>
+      <c r="G42" s="62" t="s">
         <v>48</v>
       </c>
-      <c r="H42" s="55"/>
-      <c r="I42" s="55"/>
-      <c r="J42" s="55" t="s">
+      <c r="H42" s="62"/>
+      <c r="I42" s="62"/>
+      <c r="J42" s="62" t="s">
         <v>49</v>
       </c>
-      <c r="K42" s="55"/>
-      <c r="L42" s="55"/>
+      <c r="K42" s="62"/>
+      <c r="L42" s="62"/>
       <c r="M42" s="31"/>
       <c r="N42" s="31"/>
       <c r="O42" s="31"/>
@@ -9695,21 +9707,21 @@
       <c r="K59" s="25"/>
       <c r="L59" s="24"/>
     </row>
-    <row r="60" spans="1:1021" s="32" customFormat="1" ht="25.5">
-      <c r="A60" s="68" t="s">
+    <row r="60" spans="1:1021" s="32" customFormat="1" ht="25">
+      <c r="A60" s="67" t="s">
         <v>59</v>
       </c>
-      <c r="B60" s="68"/>
-      <c r="C60" s="68"/>
-      <c r="D60" s="68"/>
-      <c r="E60" s="68"/>
-      <c r="F60" s="68"/>
-      <c r="G60" s="68"/>
-      <c r="H60" s="68"/>
-      <c r="I60" s="68"/>
-      <c r="J60" s="68"/>
-      <c r="K60" s="68"/>
-      <c r="L60" s="68"/>
+      <c r="B60" s="67"/>
+      <c r="C60" s="67"/>
+      <c r="D60" s="67"/>
+      <c r="E60" s="67"/>
+      <c r="F60" s="67"/>
+      <c r="G60" s="67"/>
+      <c r="H60" s="67"/>
+      <c r="I60" s="67"/>
+      <c r="J60" s="67"/>
+      <c r="K60" s="67"/>
+      <c r="L60" s="67"/>
       <c r="M60" s="31"/>
       <c r="N60" s="31"/>
       <c r="O60" s="31"/>
@@ -10720,27 +10732,27 @@
       <c r="AMF60" s="31"/>
       <c r="AMG60" s="31"/>
     </row>
-    <row r="61" spans="1:1021" s="32" customFormat="1" ht="25.5">
-      <c r="A61" s="56" t="s">
+    <row r="61" spans="1:1021" s="32" customFormat="1" ht="25">
+      <c r="A61" s="59" t="s">
         <v>60</v>
       </c>
-      <c r="B61" s="57"/>
-      <c r="C61" s="58"/>
-      <c r="D61" s="55" t="s">
+      <c r="B61" s="60"/>
+      <c r="C61" s="61"/>
+      <c r="D61" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="E61" s="55"/>
-      <c r="F61" s="55"/>
-      <c r="G61" s="55" t="s">
+      <c r="E61" s="62"/>
+      <c r="F61" s="62"/>
+      <c r="G61" s="62" t="s">
         <v>48</v>
       </c>
-      <c r="H61" s="55"/>
-      <c r="I61" s="55"/>
-      <c r="J61" s="55" t="s">
+      <c r="H61" s="62"/>
+      <c r="I61" s="62"/>
+      <c r="J61" s="62" t="s">
         <v>49</v>
       </c>
-      <c r="K61" s="55"/>
-      <c r="L61" s="55"/>
+      <c r="K61" s="62"/>
+      <c r="L61" s="62"/>
       <c r="M61" s="31"/>
       <c r="N61" s="31"/>
       <c r="O61" s="31"/>
@@ -12012,6 +12024,16 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A61:C61"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A22:L22"/>
+    <mergeCell ref="A41:L41"/>
+    <mergeCell ref="A60:L60"/>
+    <mergeCell ref="D61:F61"/>
+    <mergeCell ref="G61:I61"/>
+    <mergeCell ref="J61:L61"/>
+    <mergeCell ref="D42:F42"/>
+    <mergeCell ref="G42:I42"/>
     <mergeCell ref="D1:L1"/>
     <mergeCell ref="J42:L42"/>
     <mergeCell ref="D23:F23"/>
@@ -12024,16 +12046,6 @@
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A23:C23"/>
     <mergeCell ref="A42:C42"/>
-    <mergeCell ref="A61:C61"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A22:L22"/>
-    <mergeCell ref="A41:L41"/>
-    <mergeCell ref="A60:L60"/>
-    <mergeCell ref="D61:F61"/>
-    <mergeCell ref="G61:I61"/>
-    <mergeCell ref="J61:L61"/>
-    <mergeCell ref="D42:F42"/>
-    <mergeCell ref="G42:I42"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -12043,77 +12055,77 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{396D4AB3-D735-C84A-BDAA-B734A45CA873}">
   <dimension ref="A1:L46"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.5"/>
   <cols>
-    <col min="1" max="1" width="30.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="30.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.69140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.07421875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.765625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.69140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.07421875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.765625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="30.69140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.07421875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="25.5">
-      <c r="A1" s="69" t="s">
+    <row r="1" spans="1:12" ht="25">
+      <c r="A1" s="66" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-    </row>
-    <row r="2" spans="1:12" s="6" customFormat="1" ht="59.1" customHeight="1">
-      <c r="A2" s="65" t="s">
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+    </row>
+    <row r="2" spans="1:12" s="6" customFormat="1" ht="59.15" customHeight="1">
+      <c r="A2" s="68" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="66"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="66"/>
-      <c r="G2" s="66"/>
-      <c r="H2" s="66"/>
-      <c r="I2" s="67"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="70"/>
       <c r="J2" s="45"/>
       <c r="K2" s="45"/>
       <c r="L2" s="45"/>
     </row>
-    <row r="3" spans="1:12" ht="25.5">
-      <c r="A3" s="62" t="s">
+    <row r="3" spans="1:12" ht="25">
+      <c r="A3" s="63" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="63"/>
-      <c r="D3" s="63"/>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
-      <c r="G3" s="63"/>
-      <c r="H3" s="63"/>
-      <c r="I3" s="64"/>
-    </row>
-    <row r="4" spans="1:12" ht="25.5">
-      <c r="A4" s="55" t="s">
+      <c r="B3" s="64"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="64"/>
+      <c r="H3" s="64"/>
+      <c r="I3" s="65"/>
+    </row>
+    <row r="4" spans="1:12" ht="25">
+      <c r="A4" s="62" t="s">
         <v>62</v>
       </c>
-      <c r="B4" s="55"/>
-      <c r="C4" s="55"/>
-      <c r="D4" s="55" t="s">
+      <c r="B4" s="62"/>
+      <c r="C4" s="62"/>
+      <c r="D4" s="62" t="s">
         <v>63</v>
       </c>
-      <c r="E4" s="55"/>
-      <c r="F4" s="55"/>
-      <c r="G4" s="56" t="s">
+      <c r="E4" s="62"/>
+      <c r="F4" s="62"/>
+      <c r="G4" s="59" t="s">
         <v>64</v>
       </c>
-      <c r="H4" s="57"/>
-      <c r="I4" s="58"/>
+      <c r="H4" s="60"/>
+      <c r="I4" s="61"/>
     </row>
     <row r="5" spans="1:12">
       <c r="A5" s="19" t="s">
@@ -12316,35 +12328,35 @@
       <c r="H13" s="11"/>
       <c r="I13" s="19"/>
     </row>
-    <row r="14" spans="1:12" ht="25.5">
-      <c r="A14" s="62" t="s">
+    <row r="14" spans="1:12" ht="25">
+      <c r="A14" s="63" t="s">
         <v>57</v>
       </c>
-      <c r="B14" s="63"/>
-      <c r="C14" s="63"/>
-      <c r="D14" s="63"/>
-      <c r="E14" s="63"/>
-      <c r="F14" s="63"/>
-      <c r="G14" s="63"/>
-      <c r="H14" s="63"/>
-      <c r="I14" s="64"/>
-    </row>
-    <row r="15" spans="1:12" ht="25.5">
-      <c r="A15" s="55" t="s">
+      <c r="B14" s="64"/>
+      <c r="C14" s="64"/>
+      <c r="D14" s="64"/>
+      <c r="E14" s="64"/>
+      <c r="F14" s="64"/>
+      <c r="G14" s="64"/>
+      <c r="H14" s="64"/>
+      <c r="I14" s="65"/>
+    </row>
+    <row r="15" spans="1:12" ht="25">
+      <c r="A15" s="62" t="s">
         <v>62</v>
       </c>
-      <c r="B15" s="55"/>
-      <c r="C15" s="55"/>
-      <c r="D15" s="55" t="s">
+      <c r="B15" s="62"/>
+      <c r="C15" s="62"/>
+      <c r="D15" s="62" t="s">
         <v>63</v>
       </c>
-      <c r="E15" s="55"/>
-      <c r="F15" s="55"/>
-      <c r="G15" s="56" t="s">
+      <c r="E15" s="62"/>
+      <c r="F15" s="62"/>
+      <c r="G15" s="59" t="s">
         <v>64</v>
       </c>
-      <c r="H15" s="57"/>
-      <c r="I15" s="58"/>
+      <c r="H15" s="60"/>
+      <c r="I15" s="61"/>
     </row>
     <row r="16" spans="1:12">
       <c r="A16" s="19" t="s">
@@ -12547,35 +12559,35 @@
       <c r="H24" s="11"/>
       <c r="I24" s="19"/>
     </row>
-    <row r="25" spans="1:9" ht="25.5">
-      <c r="A25" s="62" t="s">
+    <row r="25" spans="1:9" ht="25">
+      <c r="A25" s="63" t="s">
         <v>58</v>
       </c>
-      <c r="B25" s="63"/>
-      <c r="C25" s="63"/>
-      <c r="D25" s="63"/>
-      <c r="E25" s="63"/>
-      <c r="F25" s="63"/>
-      <c r="G25" s="63"/>
-      <c r="H25" s="63"/>
-      <c r="I25" s="64"/>
-    </row>
-    <row r="26" spans="1:9" ht="25.5">
-      <c r="A26" s="55" t="s">
+      <c r="B25" s="64"/>
+      <c r="C25" s="64"/>
+      <c r="D25" s="64"/>
+      <c r="E25" s="64"/>
+      <c r="F25" s="64"/>
+      <c r="G25" s="64"/>
+      <c r="H25" s="64"/>
+      <c r="I25" s="65"/>
+    </row>
+    <row r="26" spans="1:9" ht="25">
+      <c r="A26" s="62" t="s">
         <v>62</v>
       </c>
-      <c r="B26" s="55"/>
-      <c r="C26" s="55"/>
-      <c r="D26" s="55" t="s">
+      <c r="B26" s="62"/>
+      <c r="C26" s="62"/>
+      <c r="D26" s="62" t="s">
         <v>63</v>
       </c>
-      <c r="E26" s="55"/>
-      <c r="F26" s="55"/>
-      <c r="G26" s="56" t="s">
+      <c r="E26" s="62"/>
+      <c r="F26" s="62"/>
+      <c r="G26" s="59" t="s">
         <v>64</v>
       </c>
-      <c r="H26" s="57"/>
-      <c r="I26" s="58"/>
+      <c r="H26" s="60"/>
+      <c r="I26" s="61"/>
     </row>
     <row r="27" spans="1:9">
       <c r="A27" s="19" t="s">
@@ -12778,35 +12790,35 @@
       <c r="H35" s="11"/>
       <c r="I35" s="19"/>
     </row>
-    <row r="36" spans="1:9" ht="25.5">
-      <c r="A36" s="62" t="s">
+    <row r="36" spans="1:9" ht="25">
+      <c r="A36" s="63" t="s">
         <v>59</v>
       </c>
-      <c r="B36" s="63"/>
-      <c r="C36" s="63"/>
-      <c r="D36" s="63"/>
-      <c r="E36" s="63"/>
-      <c r="F36" s="63"/>
-      <c r="G36" s="63"/>
-      <c r="H36" s="63"/>
-      <c r="I36" s="64"/>
-    </row>
-    <row r="37" spans="1:9" ht="25.5">
-      <c r="A37" s="55" t="s">
+      <c r="B36" s="64"/>
+      <c r="C36" s="64"/>
+      <c r="D36" s="64"/>
+      <c r="E36" s="64"/>
+      <c r="F36" s="64"/>
+      <c r="G36" s="64"/>
+      <c r="H36" s="64"/>
+      <c r="I36" s="65"/>
+    </row>
+    <row r="37" spans="1:9" ht="25">
+      <c r="A37" s="62" t="s">
         <v>62</v>
       </c>
-      <c r="B37" s="55"/>
-      <c r="C37" s="55"/>
-      <c r="D37" s="55" t="s">
+      <c r="B37" s="62"/>
+      <c r="C37" s="62"/>
+      <c r="D37" s="62" t="s">
         <v>63</v>
       </c>
-      <c r="E37" s="55"/>
-      <c r="F37" s="55"/>
-      <c r="G37" s="56" t="s">
+      <c r="E37" s="62"/>
+      <c r="F37" s="62"/>
+      <c r="G37" s="59" t="s">
         <v>64</v>
       </c>
-      <c r="H37" s="57"/>
-      <c r="I37" s="58"/>
+      <c r="H37" s="60"/>
+      <c r="I37" s="61"/>
     </row>
     <row r="38" spans="1:9">
       <c r="A38" s="19" t="s">
@@ -13011,12 +13023,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="G4:I4"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A2:I2"/>
     <mergeCell ref="A36:I36"/>
     <mergeCell ref="A37:C37"/>
     <mergeCell ref="D37:F37"/>
@@ -13029,6 +13035,12 @@
     <mergeCell ref="A26:C26"/>
     <mergeCell ref="D26:F26"/>
     <mergeCell ref="G26:I26"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="G4:I4"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -13037,21 +13049,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AMJ73"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.109375" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.07421875" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="58" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="7.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="11.109375" style="6"/>
+    <col min="2" max="3" width="7.69140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.07421875" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="11.07421875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1024" ht="25.5">
-      <c r="A1" s="49" t="s">
+    <row r="1" spans="1:1024" ht="25">
+      <c r="A1" s="50" t="s">
         <v>56</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
     </row>
     <row r="2" spans="1:1024">
       <c r="A2" s="17" t="s">
@@ -14105,13 +14117,13 @@
       <c r="AMI3" s="10"/>
       <c r="AMJ3" s="10"/>
     </row>
-    <row r="4" spans="1:1024" ht="25.5">
-      <c r="A4" s="49" t="s">
+    <row r="4" spans="1:1024" ht="25">
+      <c r="A4" s="50" t="s">
         <v>57</v>
       </c>
-      <c r="B4" s="49"/>
-      <c r="C4" s="49"/>
-      <c r="D4" s="49"/>
+      <c r="B4" s="50"/>
+      <c r="C4" s="50"/>
+      <c r="D4" s="50"/>
       <c r="G4" s="7"/>
       <c r="H4" s="7"/>
       <c r="J4" s="7"/>
@@ -15179,13 +15191,13 @@
       <c r="AMI6" s="10"/>
       <c r="AMJ6" s="10"/>
     </row>
-    <row r="7" spans="1:1024" ht="25.5">
-      <c r="A7" s="49" t="s">
+    <row r="7" spans="1:1024" ht="25">
+      <c r="A7" s="50" t="s">
         <v>58</v>
       </c>
-      <c r="B7" s="49"/>
-      <c r="C7" s="49"/>
-      <c r="D7" s="49"/>
+      <c r="B7" s="50"/>
+      <c r="C7" s="50"/>
+      <c r="D7" s="50"/>
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
       <c r="J7" s="7"/>
@@ -16245,13 +16257,13 @@
       <c r="AMI9" s="10"/>
       <c r="AMJ9" s="10"/>
     </row>
-    <row r="10" spans="1:1024" ht="25.5">
-      <c r="A10" s="49" t="s">
+    <row r="10" spans="1:1024" ht="25">
+      <c r="A10" s="50" t="s">
         <v>59</v>
       </c>
-      <c r="B10" s="49"/>
-      <c r="C10" s="49"/>
-      <c r="D10" s="49"/>
+      <c r="B10" s="50"/>
+      <c r="C10" s="50"/>
+      <c r="D10" s="50"/>
       <c r="G10" s="7"/>
       <c r="J10" s="7"/>
       <c r="K10" s="7"/>
@@ -16286,13 +16298,13 @@
       <c r="A12" s="11">
         <v>1.0668</v>
       </c>
-      <c r="B12" s="71">
+      <c r="B12" s="47">
         <v>0.42084300000000002</v>
       </c>
-      <c r="C12" s="71">
+      <c r="C12" s="47">
         <v>2.433571E-2</v>
       </c>
-      <c r="D12" s="71">
+      <c r="D12" s="47">
         <v>6.6635679999999999E-3</v>
       </c>
       <c r="E12" s="10"/>
@@ -17325,13 +17337,13 @@
       <c r="Q13" s="7"/>
       <c r="R13" s="7"/>
     </row>
-    <row r="14" spans="1:1024" ht="25.5">
-      <c r="A14" s="50" t="s">
+    <row r="14" spans="1:1024" ht="25">
+      <c r="A14" s="51" t="s">
         <v>44</v>
       </c>
-      <c r="B14" s="50"/>
-      <c r="C14" s="50"/>
-      <c r="D14" s="50"/>
+      <c r="B14" s="51"/>
+      <c r="C14" s="51"/>
+      <c r="D14" s="51"/>
       <c r="J14" s="7"/>
       <c r="K14" s="7"/>
       <c r="L14" s="7"/>
@@ -17765,21 +17777,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9E0F765-C5B1-654D-95FF-016841AE7F76}">
   <dimension ref="A1:AMJ57"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.109375" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.07421875" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="58" style="9" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="7.6640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.109375" style="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="1024" width="11.109375" style="9"/>
+    <col min="2" max="3" width="7.69140625" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.07421875" style="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="1024" width="11.07421875" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="25.5">
-      <c r="A1" s="52" t="s">
+    <row r="1" spans="1:18" ht="25">
+      <c r="A1" s="53" t="s">
         <v>56</v>
       </c>
-      <c r="B1" s="53"/>
-      <c r="C1" s="53"/>
-      <c r="D1" s="54"/>
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="55"/>
     </row>
     <row r="2" spans="1:18">
       <c r="A2" s="19" t="s">
@@ -17820,13 +17832,13 @@
       <c r="I3" s="10"/>
       <c r="O3" s="10"/>
     </row>
-    <row r="4" spans="1:18" s="9" customFormat="1" ht="25.5">
-      <c r="A4" s="52" t="s">
+    <row r="4" spans="1:18" s="9" customFormat="1" ht="25">
+      <c r="A4" s="53" t="s">
         <v>57</v>
       </c>
-      <c r="B4" s="53"/>
-      <c r="C4" s="53"/>
-      <c r="D4" s="54"/>
+      <c r="B4" s="54"/>
+      <c r="C4" s="54"/>
+      <c r="D4" s="55"/>
       <c r="E4" s="10"/>
       <c r="F4" s="10"/>
       <c r="I4" s="10"/>
@@ -17864,13 +17876,13 @@
       <c r="I6" s="10"/>
       <c r="O6" s="10"/>
     </row>
-    <row r="7" spans="1:18" s="9" customFormat="1" ht="25.5">
-      <c r="A7" s="52" t="s">
+    <row r="7" spans="1:18" s="9" customFormat="1" ht="25">
+      <c r="A7" s="53" t="s">
         <v>58</v>
       </c>
-      <c r="B7" s="53"/>
-      <c r="C7" s="53"/>
-      <c r="D7" s="54"/>
+      <c r="B7" s="54"/>
+      <c r="C7" s="54"/>
+      <c r="D7" s="55"/>
       <c r="E7" s="10"/>
       <c r="F7" s="10"/>
       <c r="G7" s="10"/>
@@ -17917,13 +17929,13 @@
       <c r="N9" s="10"/>
       <c r="O9" s="10"/>
     </row>
-    <row r="10" spans="1:18" s="9" customFormat="1" ht="25.5">
-      <c r="A10" s="52" t="s">
+    <row r="10" spans="1:18" s="9" customFormat="1" ht="25">
+      <c r="A10" s="53" t="s">
         <v>59</v>
       </c>
-      <c r="B10" s="53"/>
-      <c r="C10" s="53"/>
-      <c r="D10" s="54"/>
+      <c r="B10" s="54"/>
+      <c r="C10" s="54"/>
+      <c r="D10" s="55"/>
       <c r="E10" s="10"/>
       <c r="F10" s="10"/>
       <c r="I10" s="10"/>
@@ -17979,13 +17991,13 @@
       <c r="N13" s="10"/>
       <c r="O13" s="10"/>
     </row>
-    <row r="14" spans="1:18" s="9" customFormat="1" ht="25.5">
-      <c r="A14" s="51" t="s">
+    <row r="14" spans="1:18" s="9" customFormat="1" ht="25">
+      <c r="A14" s="52" t="s">
         <v>46</v>
       </c>
-      <c r="B14" s="51"/>
-      <c r="C14" s="51"/>
-      <c r="D14" s="51"/>
+      <c r="B14" s="52"/>
+      <c r="C14" s="52"/>
+      <c r="D14" s="52"/>
       <c r="E14" s="10"/>
       <c r="F14" s="10"/>
       <c r="G14" s="10"/>
@@ -17995,13 +18007,13 @@
       <c r="N14" s="10"/>
       <c r="O14" s="10"/>
     </row>
-    <row r="15" spans="1:18" s="9" customFormat="1" ht="25.5">
-      <c r="A15" s="51" t="s">
+    <row r="15" spans="1:18" s="9" customFormat="1" ht="25">
+      <c r="A15" s="52" t="s">
         <v>44</v>
       </c>
-      <c r="B15" s="51"/>
-      <c r="C15" s="51"/>
-      <c r="D15" s="51"/>
+      <c r="B15" s="52"/>
+      <c r="C15" s="52"/>
+      <c r="D15" s="52"/>
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
       <c r="G15" s="10"/>
@@ -18449,21 +18461,21 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:AMJ69"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.109375" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.07421875" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="58" style="9" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="7.6640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.109375" style="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="1024" width="11.109375" style="9"/>
+    <col min="2" max="3" width="7.69140625" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.07421875" style="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="1024" width="11.07421875" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="25.5">
-      <c r="A1" s="52" t="s">
+    <row r="1" spans="1:18" ht="25">
+      <c r="A1" s="53" t="s">
         <v>56</v>
       </c>
-      <c r="B1" s="53"/>
-      <c r="C1" s="53"/>
-      <c r="D1" s="54"/>
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="55"/>
     </row>
     <row r="2" spans="1:18">
       <c r="A2" s="19" t="s">
@@ -18549,13 +18561,13 @@
       <c r="I6" s="10"/>
       <c r="O6" s="10"/>
     </row>
-    <row r="7" spans="1:18" ht="25.5">
-      <c r="A7" s="52" t="s">
+    <row r="7" spans="1:18" ht="25">
+      <c r="A7" s="53" t="s">
         <v>57</v>
       </c>
-      <c r="B7" s="53"/>
-      <c r="C7" s="53"/>
-      <c r="D7" s="54"/>
+      <c r="B7" s="54"/>
+      <c r="C7" s="54"/>
+      <c r="D7" s="55"/>
       <c r="E7" s="10"/>
       <c r="F7" s="10"/>
       <c r="I7" s="10"/>
@@ -18635,13 +18647,13 @@
       <c r="I12" s="10"/>
       <c r="O12" s="10"/>
     </row>
-    <row r="13" spans="1:18" ht="25.5">
-      <c r="A13" s="52" t="s">
+    <row r="13" spans="1:18" ht="25">
+      <c r="A13" s="53" t="s">
         <v>58</v>
       </c>
-      <c r="B13" s="53"/>
-      <c r="C13" s="53"/>
-      <c r="D13" s="54"/>
+      <c r="B13" s="54"/>
+      <c r="C13" s="54"/>
+      <c r="D13" s="55"/>
       <c r="E13" s="10"/>
       <c r="F13" s="10"/>
       <c r="G13" s="10"/>
@@ -18732,13 +18744,13 @@
       <c r="N18" s="10"/>
       <c r="O18" s="10"/>
     </row>
-    <row r="19" spans="1:15" ht="25.5">
-      <c r="A19" s="52" t="s">
+    <row r="19" spans="1:15" ht="25">
+      <c r="A19" s="53" t="s">
         <v>59</v>
       </c>
-      <c r="B19" s="53"/>
-      <c r="C19" s="53"/>
-      <c r="D19" s="54"/>
+      <c r="B19" s="54"/>
+      <c r="C19" s="54"/>
+      <c r="D19" s="55"/>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
       <c r="I19" s="10"/>
@@ -18840,13 +18852,13 @@
       <c r="N25" s="10"/>
       <c r="O25" s="10"/>
     </row>
-    <row r="26" spans="1:15" ht="25.5">
-      <c r="A26" s="51" t="s">
+    <row r="26" spans="1:15" ht="25">
+      <c r="A26" s="52" t="s">
         <v>46</v>
       </c>
-      <c r="B26" s="51"/>
-      <c r="C26" s="51"/>
-      <c r="D26" s="51"/>
+      <c r="B26" s="52"/>
+      <c r="C26" s="52"/>
+      <c r="D26" s="52"/>
       <c r="E26" s="10"/>
       <c r="F26" s="10"/>
       <c r="G26" s="10"/>
@@ -18856,13 +18868,13 @@
       <c r="N26" s="10"/>
       <c r="O26" s="10"/>
     </row>
-    <row r="27" spans="1:15" ht="25.5">
-      <c r="A27" s="51" t="s">
+    <row r="27" spans="1:15" ht="25">
+      <c r="A27" s="52" t="s">
         <v>44</v>
       </c>
-      <c r="B27" s="51"/>
-      <c r="C27" s="51"/>
-      <c r="D27" s="51"/>
+      <c r="B27" s="52"/>
+      <c r="C27" s="52"/>
+      <c r="D27" s="52"/>
       <c r="E27" s="10"/>
       <c r="F27" s="10"/>
       <c r="G27" s="10"/>
@@ -19310,80 +19322,80 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EA0DC49-B228-6142-89A2-F876D0182B62}">
   <dimension ref="A1:M17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.5"/>
   <cols>
-    <col min="1" max="1" width="30.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.77734375" style="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.69140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.07421875" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.765625" style="6" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="25" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.77734375" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.07421875" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.765625" style="6" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="25" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.77734375" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.07421875" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.765625" style="6" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="25" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="23.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="20.77734375" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23.07421875" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20.765625" style="6" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="25" style="6" bestFit="1" customWidth="1"/>
     <col min="14" max="16384" width="11" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="25.5">
-      <c r="A1" s="59" t="s">
+    <row r="1" spans="1:13" ht="25">
+      <c r="A1" s="56" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="60"/>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="61"/>
-    </row>
-    <row r="2" spans="1:13" ht="25.5">
-      <c r="A2" s="55" t="s">
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
+      <c r="H1" s="57"/>
+      <c r="I1" s="57"/>
+      <c r="J1" s="57"/>
+      <c r="K1" s="57"/>
+      <c r="L1" s="57"/>
+      <c r="M1" s="58"/>
+    </row>
+    <row r="2" spans="1:13" ht="25">
+      <c r="A2" s="62" t="s">
         <v>56</v>
       </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="J2" s="55"/>
-      <c r="K2" s="55"/>
-      <c r="L2" s="55"/>
-      <c r="M2" s="55"/>
-    </row>
-    <row r="3" spans="1:13" ht="25.5">
-      <c r="A3" s="55" t="s">
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="62"/>
+      <c r="L2" s="62"/>
+      <c r="M2" s="62"/>
+    </row>
+    <row r="3" spans="1:13" ht="25">
+      <c r="A3" s="62" t="s">
         <v>60</v>
       </c>
-      <c r="B3" s="55"/>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55" t="s">
+      <c r="B3" s="62"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="F3" s="55"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="56" t="s">
+      <c r="F3" s="62"/>
+      <c r="G3" s="62"/>
+      <c r="H3" s="59" t="s">
         <v>48</v>
       </c>
-      <c r="I3" s="57"/>
-      <c r="J3" s="58"/>
-      <c r="K3" s="56" t="s">
+      <c r="I3" s="60"/>
+      <c r="J3" s="61"/>
+      <c r="K3" s="59" t="s">
         <v>49</v>
       </c>
-      <c r="L3" s="57"/>
-      <c r="M3" s="58"/>
+      <c r="L3" s="60"/>
+      <c r="M3" s="61"/>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="17"/>
@@ -19445,45 +19457,45 @@
         <v>9.6127163999999987E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="25.5">
-      <c r="A6" s="62" t="s">
+    <row r="6" spans="1:13" ht="25">
+      <c r="A6" s="63" t="s">
         <v>57</v>
       </c>
-      <c r="B6" s="63"/>
-      <c r="C6" s="63"/>
-      <c r="D6" s="63"/>
-      <c r="E6" s="63"/>
-      <c r="F6" s="63"/>
-      <c r="G6" s="63"/>
-      <c r="H6" s="63"/>
-      <c r="I6" s="63"/>
-      <c r="J6" s="63"/>
-      <c r="K6" s="63"/>
-      <c r="L6" s="63"/>
-      <c r="M6" s="64"/>
-    </row>
-    <row r="7" spans="1:13" ht="25.5">
-      <c r="A7" s="55" t="s">
+      <c r="B6" s="64"/>
+      <c r="C6" s="64"/>
+      <c r="D6" s="64"/>
+      <c r="E6" s="64"/>
+      <c r="F6" s="64"/>
+      <c r="G6" s="64"/>
+      <c r="H6" s="64"/>
+      <c r="I6" s="64"/>
+      <c r="J6" s="64"/>
+      <c r="K6" s="64"/>
+      <c r="L6" s="64"/>
+      <c r="M6" s="65"/>
+    </row>
+    <row r="7" spans="1:13" ht="25">
+      <c r="A7" s="62" t="s">
         <v>60</v>
       </c>
-      <c r="B7" s="55"/>
-      <c r="C7" s="55"/>
-      <c r="D7" s="55"/>
-      <c r="E7" s="55" t="s">
+      <c r="B7" s="62"/>
+      <c r="C7" s="62"/>
+      <c r="D7" s="62"/>
+      <c r="E7" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="F7" s="55"/>
-      <c r="G7" s="55"/>
-      <c r="H7" s="56" t="s">
+      <c r="F7" s="62"/>
+      <c r="G7" s="62"/>
+      <c r="H7" s="59" t="s">
         <v>48</v>
       </c>
-      <c r="I7" s="57"/>
-      <c r="J7" s="58"/>
-      <c r="K7" s="56" t="s">
+      <c r="I7" s="60"/>
+      <c r="J7" s="61"/>
+      <c r="K7" s="59" t="s">
         <v>49</v>
       </c>
-      <c r="L7" s="57"/>
-      <c r="M7" s="58"/>
+      <c r="L7" s="60"/>
+      <c r="M7" s="61"/>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="17"/>
@@ -19540,50 +19552,52 @@
       <c r="K9" s="25">
         <v>0.11529621600000001</v>
       </c>
-      <c r="L9" s="25"/>
+      <c r="L9" s="25">
+        <v>5.5062251999999999E-2</v>
+      </c>
       <c r="M9" s="25">
         <v>9.6979218000000002E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="25.5">
-      <c r="A10" s="55" t="s">
+    <row r="10" spans="1:13" ht="25">
+      <c r="A10" s="62" t="s">
         <v>58</v>
       </c>
-      <c r="B10" s="55"/>
-      <c r="C10" s="55"/>
-      <c r="D10" s="55"/>
-      <c r="E10" s="55"/>
-      <c r="F10" s="55"/>
-      <c r="G10" s="55"/>
-      <c r="H10" s="55"/>
-      <c r="I10" s="55"/>
-      <c r="J10" s="55"/>
-      <c r="K10" s="55"/>
-      <c r="L10" s="55"/>
-      <c r="M10" s="55"/>
-    </row>
-    <row r="11" spans="1:13" ht="25.5">
-      <c r="A11" s="55" t="s">
+      <c r="B10" s="62"/>
+      <c r="C10" s="62"/>
+      <c r="D10" s="62"/>
+      <c r="E10" s="62"/>
+      <c r="F10" s="62"/>
+      <c r="G10" s="62"/>
+      <c r="H10" s="62"/>
+      <c r="I10" s="62"/>
+      <c r="J10" s="62"/>
+      <c r="K10" s="62"/>
+      <c r="L10" s="62"/>
+      <c r="M10" s="62"/>
+    </row>
+    <row r="11" spans="1:13" ht="25">
+      <c r="A11" s="62" t="s">
         <v>60</v>
       </c>
-      <c r="B11" s="55"/>
-      <c r="C11" s="55"/>
-      <c r="D11" s="55"/>
-      <c r="E11" s="55" t="s">
+      <c r="B11" s="62"/>
+      <c r="C11" s="62"/>
+      <c r="D11" s="62"/>
+      <c r="E11" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="55"/>
-      <c r="G11" s="55"/>
-      <c r="H11" s="56" t="s">
+      <c r="F11" s="62"/>
+      <c r="G11" s="62"/>
+      <c r="H11" s="59" t="s">
         <v>48</v>
       </c>
-      <c r="I11" s="57"/>
-      <c r="J11" s="58"/>
-      <c r="K11" s="56" t="s">
+      <c r="I11" s="60"/>
+      <c r="J11" s="61"/>
+      <c r="K11" s="59" t="s">
         <v>49</v>
       </c>
-      <c r="L11" s="57"/>
-      <c r="M11" s="58"/>
+      <c r="L11" s="60"/>
+      <c r="M11" s="61"/>
     </row>
     <row r="12" spans="1:13">
       <c r="A12" s="17"/>
@@ -19641,45 +19655,45 @@
       <c r="L13" s="41"/>
       <c r="M13" s="41"/>
     </row>
-    <row r="14" spans="1:13" ht="25.5">
-      <c r="A14" s="55" t="s">
+    <row r="14" spans="1:13" ht="25">
+      <c r="A14" s="62" t="s">
         <v>59</v>
       </c>
-      <c r="B14" s="55"/>
-      <c r="C14" s="55"/>
-      <c r="D14" s="55"/>
-      <c r="E14" s="55"/>
-      <c r="F14" s="55"/>
-      <c r="G14" s="55"/>
-      <c r="H14" s="55"/>
-      <c r="I14" s="55"/>
-      <c r="J14" s="55"/>
-      <c r="K14" s="55"/>
-      <c r="L14" s="55"/>
-      <c r="M14" s="55"/>
-    </row>
-    <row r="15" spans="1:13" ht="25.5">
-      <c r="A15" s="55" t="s">
+      <c r="B14" s="62"/>
+      <c r="C14" s="62"/>
+      <c r="D14" s="62"/>
+      <c r="E14" s="62"/>
+      <c r="F14" s="62"/>
+      <c r="G14" s="62"/>
+      <c r="H14" s="62"/>
+      <c r="I14" s="62"/>
+      <c r="J14" s="62"/>
+      <c r="K14" s="62"/>
+      <c r="L14" s="62"/>
+      <c r="M14" s="62"/>
+    </row>
+    <row r="15" spans="1:13" ht="25">
+      <c r="A15" s="62" t="s">
         <v>60</v>
       </c>
-      <c r="B15" s="55"/>
-      <c r="C15" s="55"/>
-      <c r="D15" s="55"/>
-      <c r="E15" s="55" t="s">
+      <c r="B15" s="62"/>
+      <c r="C15" s="62"/>
+      <c r="D15" s="62"/>
+      <c r="E15" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="F15" s="55"/>
-      <c r="G15" s="55"/>
-      <c r="H15" s="56" t="s">
+      <c r="F15" s="62"/>
+      <c r="G15" s="62"/>
+      <c r="H15" s="59" t="s">
         <v>48</v>
       </c>
-      <c r="I15" s="57"/>
-      <c r="J15" s="58"/>
-      <c r="K15" s="56" t="s">
+      <c r="I15" s="60"/>
+      <c r="J15" s="61"/>
+      <c r="K15" s="59" t="s">
         <v>49</v>
       </c>
-      <c r="L15" s="57"/>
-      <c r="M15" s="58"/>
+      <c r="L15" s="60"/>
+      <c r="M15" s="61"/>
     </row>
     <row r="16" spans="1:13">
       <c r="A16" s="17"/>
@@ -19743,6 +19757,16 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="A14:M14"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="H15:J15"/>
+    <mergeCell ref="K15:M15"/>
+    <mergeCell ref="A10:M10"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="K11:M11"/>
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="K3:M3"/>
     <mergeCell ref="A2:M2"/>
@@ -19754,16 +19778,6 @@
     <mergeCell ref="E3:G3"/>
     <mergeCell ref="H3:J3"/>
     <mergeCell ref="K7:M7"/>
-    <mergeCell ref="A10:M10"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="E11:G11"/>
-    <mergeCell ref="H11:J11"/>
-    <mergeCell ref="K11:M11"/>
-    <mergeCell ref="A14:M14"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="E15:G15"/>
-    <mergeCell ref="H15:J15"/>
-    <mergeCell ref="K15:M15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -19772,93 +19786,93 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:Q78"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.5"/>
   <cols>
-    <col min="1" max="1" width="30.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.77734375" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.77734375" style="10" customWidth="1"/>
-    <col min="7" max="7" width="30.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.77734375" style="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="30.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="23.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.77734375" style="6" bestFit="1" customWidth="1"/>
-    <col min="13" max="17" width="13.6640625" style="6" customWidth="1"/>
+    <col min="1" max="1" width="30.69140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.07421875" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.765625" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.69140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.07421875" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.765625" style="10" customWidth="1"/>
+    <col min="7" max="7" width="30.69140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.07421875" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.765625" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="30.69140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23.07421875" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.765625" style="6" bestFit="1" customWidth="1"/>
+    <col min="13" max="17" width="13.69140625" style="6" customWidth="1"/>
     <col min="18" max="16384" width="11" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="25.5">
-      <c r="A1" s="69" t="s">
+    <row r="1" spans="1:17" ht="25">
+      <c r="A1" s="66" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
-      <c r="L1" s="69"/>
-    </row>
-    <row r="2" spans="1:17" ht="59.1" customHeight="1">
-      <c r="A2" s="65" t="s">
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="66"/>
+      <c r="L1" s="66"/>
+    </row>
+    <row r="2" spans="1:17" ht="59.15" customHeight="1">
+      <c r="A2" s="68" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="66"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="66"/>
-      <c r="G2" s="66"/>
-      <c r="H2" s="66"/>
-      <c r="I2" s="66"/>
-      <c r="J2" s="66"/>
-      <c r="K2" s="66"/>
-      <c r="L2" s="67"/>
-    </row>
-    <row r="3" spans="1:17" s="27" customFormat="1" ht="25.5">
-      <c r="A3" s="55" t="s">
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="70"/>
+    </row>
+    <row r="3" spans="1:17" s="27" customFormat="1" ht="25">
+      <c r="A3" s="62" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="55"/>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="55"/>
-      <c r="I3" s="55"/>
-      <c r="J3" s="55"/>
-      <c r="K3" s="55"/>
-      <c r="L3" s="55"/>
-    </row>
-    <row r="4" spans="1:17" s="27" customFormat="1" ht="25.5">
-      <c r="A4" s="55" t="s">
+      <c r="B3" s="62"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
+      <c r="G3" s="62"/>
+      <c r="H3" s="62"/>
+      <c r="I3" s="62"/>
+      <c r="J3" s="62"/>
+      <c r="K3" s="62"/>
+      <c r="L3" s="62"/>
+    </row>
+    <row r="4" spans="1:17" s="27" customFormat="1" ht="25">
+      <c r="A4" s="62" t="s">
         <v>60</v>
       </c>
-      <c r="B4" s="55"/>
-      <c r="C4" s="55"/>
-      <c r="D4" s="55" t="s">
+      <c r="B4" s="62"/>
+      <c r="C4" s="62"/>
+      <c r="D4" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="E4" s="55"/>
-      <c r="F4" s="55"/>
-      <c r="G4" s="55" t="s">
+      <c r="E4" s="62"/>
+      <c r="F4" s="62"/>
+      <c r="G4" s="62" t="s">
         <v>48</v>
       </c>
-      <c r="H4" s="55"/>
-      <c r="I4" s="55"/>
-      <c r="J4" s="55" t="s">
+      <c r="H4" s="62"/>
+      <c r="I4" s="62"/>
+      <c r="J4" s="62" t="s">
         <v>49</v>
       </c>
-      <c r="K4" s="55"/>
-      <c r="L4" s="55"/>
+      <c r="K4" s="62"/>
+      <c r="L4" s="62"/>
       <c r="N4" s="18"/>
       <c r="O4" s="18"/>
       <c r="P4" s="18"/>
@@ -20237,47 +20251,47 @@
       <c r="P21" s="7"/>
       <c r="Q21" s="7"/>
     </row>
-    <row r="22" spans="1:17" s="27" customFormat="1" ht="25.5">
-      <c r="A22" s="68" t="s">
+    <row r="22" spans="1:17" s="27" customFormat="1" ht="25">
+      <c r="A22" s="67" t="s">
         <v>57</v>
       </c>
-      <c r="B22" s="68"/>
-      <c r="C22" s="68"/>
-      <c r="D22" s="68"/>
-      <c r="E22" s="68"/>
-      <c r="F22" s="68"/>
-      <c r="G22" s="68"/>
-      <c r="H22" s="68"/>
-      <c r="I22" s="68"/>
-      <c r="J22" s="68"/>
-      <c r="K22" s="68"/>
-      <c r="L22" s="68"/>
+      <c r="B22" s="67"/>
+      <c r="C22" s="67"/>
+      <c r="D22" s="67"/>
+      <c r="E22" s="67"/>
+      <c r="F22" s="67"/>
+      <c r="G22" s="67"/>
+      <c r="H22" s="67"/>
+      <c r="I22" s="67"/>
+      <c r="J22" s="67"/>
+      <c r="K22" s="67"/>
+      <c r="L22" s="67"/>
       <c r="M22" s="28"/>
       <c r="O22" s="29"/>
       <c r="P22" s="29"/>
       <c r="Q22" s="29"/>
     </row>
-    <row r="23" spans="1:17" s="27" customFormat="1" ht="25.5">
-      <c r="A23" s="55" t="s">
+    <row r="23" spans="1:17" s="27" customFormat="1" ht="25">
+      <c r="A23" s="62" t="s">
         <v>60</v>
       </c>
-      <c r="B23" s="55"/>
-      <c r="C23" s="55"/>
-      <c r="D23" s="55" t="s">
+      <c r="B23" s="62"/>
+      <c r="C23" s="62"/>
+      <c r="D23" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="E23" s="55"/>
-      <c r="F23" s="55"/>
-      <c r="G23" s="55" t="s">
+      <c r="E23" s="62"/>
+      <c r="F23" s="62"/>
+      <c r="G23" s="62" t="s">
         <v>48</v>
       </c>
-      <c r="H23" s="55"/>
-      <c r="I23" s="55"/>
-      <c r="J23" s="55" t="s">
+      <c r="H23" s="62"/>
+      <c r="I23" s="62"/>
+      <c r="J23" s="62" t="s">
         <v>49</v>
       </c>
-      <c r="K23" s="55"/>
-      <c r="L23" s="55"/>
+      <c r="K23" s="62"/>
+      <c r="L23" s="62"/>
       <c r="O23" s="29"/>
       <c r="P23" s="29"/>
       <c r="Q23" s="29"/>
@@ -20642,46 +20656,46 @@
       <c r="P40" s="7"/>
       <c r="Q40" s="7"/>
     </row>
-    <row r="41" spans="1:17" s="27" customFormat="1" ht="25.5">
-      <c r="A41" s="68" t="s">
+    <row r="41" spans="1:17" s="27" customFormat="1" ht="25">
+      <c r="A41" s="67" t="s">
         <v>58</v>
       </c>
-      <c r="B41" s="68"/>
-      <c r="C41" s="68"/>
-      <c r="D41" s="68"/>
-      <c r="E41" s="68"/>
-      <c r="F41" s="68"/>
-      <c r="G41" s="68"/>
-      <c r="H41" s="68"/>
-      <c r="I41" s="68"/>
-      <c r="J41" s="68"/>
-      <c r="K41" s="68"/>
-      <c r="L41" s="68"/>
+      <c r="B41" s="67"/>
+      <c r="C41" s="67"/>
+      <c r="D41" s="67"/>
+      <c r="E41" s="67"/>
+      <c r="F41" s="67"/>
+      <c r="G41" s="67"/>
+      <c r="H41" s="67"/>
+      <c r="I41" s="67"/>
+      <c r="J41" s="67"/>
+      <c r="K41" s="67"/>
+      <c r="L41" s="67"/>
       <c r="O41" s="29"/>
       <c r="P41" s="29"/>
       <c r="Q41" s="29"/>
     </row>
-    <row r="42" spans="1:17" s="27" customFormat="1" ht="25.5">
-      <c r="A42" s="55" t="s">
+    <row r="42" spans="1:17" s="27" customFormat="1" ht="25">
+      <c r="A42" s="62" t="s">
         <v>60</v>
       </c>
-      <c r="B42" s="55"/>
-      <c r="C42" s="55"/>
-      <c r="D42" s="55" t="s">
+      <c r="B42" s="62"/>
+      <c r="C42" s="62"/>
+      <c r="D42" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="E42" s="55"/>
-      <c r="F42" s="55"/>
-      <c r="G42" s="55" t="s">
+      <c r="E42" s="62"/>
+      <c r="F42" s="62"/>
+      <c r="G42" s="62" t="s">
         <v>48</v>
       </c>
-      <c r="H42" s="55"/>
-      <c r="I42" s="55"/>
-      <c r="J42" s="55" t="s">
+      <c r="H42" s="62"/>
+      <c r="I42" s="62"/>
+      <c r="J42" s="62" t="s">
         <v>49</v>
       </c>
-      <c r="K42" s="55"/>
-      <c r="L42" s="55"/>
+      <c r="K42" s="62"/>
+      <c r="L42" s="62"/>
     </row>
     <row r="43" spans="1:17">
       <c r="A43" s="19" t="s">
@@ -20992,43 +21006,43 @@
       <c r="K59" s="25"/>
       <c r="L59" s="26"/>
     </row>
-    <row r="60" spans="1:12" s="27" customFormat="1" ht="25.5">
-      <c r="A60" s="55" t="s">
+    <row r="60" spans="1:12" s="27" customFormat="1" ht="25">
+      <c r="A60" s="62" t="s">
         <v>59</v>
       </c>
-      <c r="B60" s="55"/>
-      <c r="C60" s="55"/>
-      <c r="D60" s="55"/>
-      <c r="E60" s="55"/>
-      <c r="F60" s="55"/>
-      <c r="G60" s="55"/>
-      <c r="H60" s="55"/>
-      <c r="I60" s="55"/>
-      <c r="J60" s="55"/>
-      <c r="K60" s="55"/>
-      <c r="L60" s="55"/>
-    </row>
-    <row r="61" spans="1:12" s="27" customFormat="1" ht="25.5">
-      <c r="A61" s="55" t="s">
+      <c r="B60" s="62"/>
+      <c r="C60" s="62"/>
+      <c r="D60" s="62"/>
+      <c r="E60" s="62"/>
+      <c r="F60" s="62"/>
+      <c r="G60" s="62"/>
+      <c r="H60" s="62"/>
+      <c r="I60" s="62"/>
+      <c r="J60" s="62"/>
+      <c r="K60" s="62"/>
+      <c r="L60" s="62"/>
+    </row>
+    <row r="61" spans="1:12" s="27" customFormat="1" ht="25">
+      <c r="A61" s="62" t="s">
         <v>60</v>
       </c>
-      <c r="B61" s="55"/>
-      <c r="C61" s="55"/>
-      <c r="D61" s="55" t="s">
+      <c r="B61" s="62"/>
+      <c r="C61" s="62"/>
+      <c r="D61" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="E61" s="55"/>
-      <c r="F61" s="55"/>
-      <c r="G61" s="55" t="s">
+      <c r="E61" s="62"/>
+      <c r="F61" s="62"/>
+      <c r="G61" s="62" t="s">
         <v>48</v>
       </c>
-      <c r="H61" s="55"/>
-      <c r="I61" s="55"/>
-      <c r="J61" s="55" t="s">
+      <c r="H61" s="62"/>
+      <c r="I61" s="62"/>
+      <c r="J61" s="62" t="s">
         <v>49</v>
       </c>
-      <c r="K61" s="55"/>
-      <c r="L61" s="55"/>
+      <c r="K61" s="62"/>
+      <c r="L61" s="62"/>
     </row>
     <row r="62" spans="1:12">
       <c r="A62" s="19" t="s">
@@ -21341,6 +21355,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A61:C61"/>
+    <mergeCell ref="A41:L41"/>
+    <mergeCell ref="A60:L60"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A3:L3"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A23:C23"/>
     <mergeCell ref="A42:C42"/>
@@ -21357,12 +21377,6 @@
     <mergeCell ref="D42:F42"/>
     <mergeCell ref="G42:I42"/>
     <mergeCell ref="J42:L42"/>
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A61:C61"/>
-    <mergeCell ref="A41:L41"/>
-    <mergeCell ref="A60:L60"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A3:L3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -21372,80 +21386,80 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63424B91-982A-6F4D-9CA3-A2EB040E3D0E}">
   <dimension ref="A1:M17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.5"/>
   <cols>
-    <col min="1" max="1" width="30.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.77734375" style="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.69140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.07421875" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.765625" style="6" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="25" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.77734375" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.07421875" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.765625" style="6" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="25" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.77734375" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.07421875" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.765625" style="6" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="25" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="23.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="20.77734375" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23.07421875" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20.765625" style="6" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="25" style="6" bestFit="1" customWidth="1"/>
     <col min="14" max="16384" width="11" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="25.5">
-      <c r="A1" s="59" t="s">
+    <row r="1" spans="1:13" ht="25">
+      <c r="A1" s="56" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="60"/>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="61"/>
-    </row>
-    <row r="2" spans="1:13" ht="25.5">
-      <c r="A2" s="55" t="s">
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
+      <c r="H1" s="57"/>
+      <c r="I1" s="57"/>
+      <c r="J1" s="57"/>
+      <c r="K1" s="57"/>
+      <c r="L1" s="57"/>
+      <c r="M1" s="58"/>
+    </row>
+    <row r="2" spans="1:13" ht="25">
+      <c r="A2" s="62" t="s">
         <v>56</v>
       </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="J2" s="55"/>
-      <c r="K2" s="55"/>
-      <c r="L2" s="55"/>
-      <c r="M2" s="55"/>
-    </row>
-    <row r="3" spans="1:13" ht="25.5">
-      <c r="A3" s="55" t="s">
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="62"/>
+      <c r="L2" s="62"/>
+      <c r="M2" s="62"/>
+    </row>
+    <row r="3" spans="1:13" ht="25">
+      <c r="A3" s="62" t="s">
         <v>60</v>
       </c>
-      <c r="B3" s="55"/>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55" t="s">
+      <c r="B3" s="62"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="F3" s="55"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="56" t="s">
+      <c r="F3" s="62"/>
+      <c r="G3" s="62"/>
+      <c r="H3" s="59" t="s">
         <v>48</v>
       </c>
-      <c r="I3" s="57"/>
-      <c r="J3" s="58"/>
-      <c r="K3" s="56" t="s">
+      <c r="I3" s="60"/>
+      <c r="J3" s="61"/>
+      <c r="K3" s="59" t="s">
         <v>49</v>
       </c>
-      <c r="L3" s="57"/>
-      <c r="M3" s="58"/>
+      <c r="L3" s="60"/>
+      <c r="M3" s="61"/>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="17"/>
@@ -21507,45 +21521,45 @@
         <v>1.1565640800000001E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="25.5">
-      <c r="A6" s="62" t="s">
+    <row r="6" spans="1:13" ht="25">
+      <c r="A6" s="63" t="s">
         <v>57</v>
       </c>
-      <c r="B6" s="63"/>
-      <c r="C6" s="63"/>
-      <c r="D6" s="63"/>
-      <c r="E6" s="63"/>
-      <c r="F6" s="63"/>
-      <c r="G6" s="63"/>
-      <c r="H6" s="63"/>
-      <c r="I6" s="63"/>
-      <c r="J6" s="63"/>
-      <c r="K6" s="63"/>
-      <c r="L6" s="63"/>
-      <c r="M6" s="64"/>
-    </row>
-    <row r="7" spans="1:13" ht="25.5">
-      <c r="A7" s="55" t="s">
+      <c r="B6" s="64"/>
+      <c r="C6" s="64"/>
+      <c r="D6" s="64"/>
+      <c r="E6" s="64"/>
+      <c r="F6" s="64"/>
+      <c r="G6" s="64"/>
+      <c r="H6" s="64"/>
+      <c r="I6" s="64"/>
+      <c r="J6" s="64"/>
+      <c r="K6" s="64"/>
+      <c r="L6" s="64"/>
+      <c r="M6" s="65"/>
+    </row>
+    <row r="7" spans="1:13" ht="25">
+      <c r="A7" s="62" t="s">
         <v>60</v>
       </c>
-      <c r="B7" s="55"/>
-      <c r="C7" s="55"/>
-      <c r="D7" s="55"/>
-      <c r="E7" s="55" t="s">
+      <c r="B7" s="62"/>
+      <c r="C7" s="62"/>
+      <c r="D7" s="62"/>
+      <c r="E7" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="F7" s="55"/>
-      <c r="G7" s="55"/>
-      <c r="H7" s="56" t="s">
+      <c r="F7" s="62"/>
+      <c r="G7" s="62"/>
+      <c r="H7" s="59" t="s">
         <v>48</v>
       </c>
-      <c r="I7" s="57"/>
-      <c r="J7" s="58"/>
-      <c r="K7" s="56" t="s">
+      <c r="I7" s="60"/>
+      <c r="J7" s="61"/>
+      <c r="K7" s="59" t="s">
         <v>49</v>
       </c>
-      <c r="L7" s="57"/>
-      <c r="M7" s="58"/>
+      <c r="L7" s="60"/>
+      <c r="M7" s="61"/>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="17"/>
@@ -21602,50 +21616,52 @@
       <c r="K9" s="11">
         <v>0.11506248599999999</v>
       </c>
-      <c r="L9" s="34"/>
+      <c r="L9" s="72">
+        <v>5.5776881999999993E-2</v>
+      </c>
       <c r="M9" s="11">
         <v>1.1700481800000001E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="25.5">
-      <c r="A10" s="55" t="s">
+    <row r="10" spans="1:13" ht="25">
+      <c r="A10" s="62" t="s">
         <v>58</v>
       </c>
-      <c r="B10" s="55"/>
-      <c r="C10" s="55"/>
-      <c r="D10" s="55"/>
-      <c r="E10" s="55"/>
-      <c r="F10" s="55"/>
-      <c r="G10" s="55"/>
-      <c r="H10" s="55"/>
-      <c r="I10" s="55"/>
-      <c r="J10" s="55"/>
-      <c r="K10" s="55"/>
-      <c r="L10" s="55"/>
-      <c r="M10" s="55"/>
-    </row>
-    <row r="11" spans="1:13" ht="25.5">
-      <c r="A11" s="55" t="s">
+      <c r="B10" s="62"/>
+      <c r="C10" s="62"/>
+      <c r="D10" s="62"/>
+      <c r="E10" s="62"/>
+      <c r="F10" s="62"/>
+      <c r="G10" s="62"/>
+      <c r="H10" s="62"/>
+      <c r="I10" s="62"/>
+      <c r="J10" s="62"/>
+      <c r="K10" s="62"/>
+      <c r="L10" s="62"/>
+      <c r="M10" s="62"/>
+    </row>
+    <row r="11" spans="1:13" ht="25">
+      <c r="A11" s="62" t="s">
         <v>60</v>
       </c>
-      <c r="B11" s="55"/>
-      <c r="C11" s="55"/>
-      <c r="D11" s="55"/>
-      <c r="E11" s="55" t="s">
+      <c r="B11" s="62"/>
+      <c r="C11" s="62"/>
+      <c r="D11" s="62"/>
+      <c r="E11" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="55"/>
-      <c r="G11" s="55"/>
-      <c r="H11" s="56" t="s">
+      <c r="F11" s="62"/>
+      <c r="G11" s="62"/>
+      <c r="H11" s="59" t="s">
         <v>48</v>
       </c>
-      <c r="I11" s="57"/>
-      <c r="J11" s="58"/>
-      <c r="K11" s="56" t="s">
+      <c r="I11" s="60"/>
+      <c r="J11" s="61"/>
+      <c r="K11" s="59" t="s">
         <v>49</v>
       </c>
-      <c r="L11" s="57"/>
-      <c r="M11" s="58"/>
+      <c r="L11" s="60"/>
+      <c r="M11" s="61"/>
     </row>
     <row r="12" spans="1:13">
       <c r="A12" s="17"/>
@@ -21703,45 +21719,45 @@
       <c r="L13" s="34"/>
       <c r="M13" s="11"/>
     </row>
-    <row r="14" spans="1:13" ht="25.5">
-      <c r="A14" s="55" t="s">
+    <row r="14" spans="1:13" ht="25">
+      <c r="A14" s="62" t="s">
         <v>59</v>
       </c>
-      <c r="B14" s="55"/>
-      <c r="C14" s="55"/>
-      <c r="D14" s="55"/>
-      <c r="E14" s="55"/>
-      <c r="F14" s="55"/>
-      <c r="G14" s="55"/>
-      <c r="H14" s="55"/>
-      <c r="I14" s="55"/>
-      <c r="J14" s="55"/>
-      <c r="K14" s="55"/>
-      <c r="L14" s="55"/>
-      <c r="M14" s="55"/>
-    </row>
-    <row r="15" spans="1:13" ht="25.5">
-      <c r="A15" s="55" t="s">
+      <c r="B14" s="62"/>
+      <c r="C14" s="62"/>
+      <c r="D14" s="62"/>
+      <c r="E14" s="62"/>
+      <c r="F14" s="62"/>
+      <c r="G14" s="62"/>
+      <c r="H14" s="62"/>
+      <c r="I14" s="62"/>
+      <c r="J14" s="62"/>
+      <c r="K14" s="62"/>
+      <c r="L14" s="62"/>
+      <c r="M14" s="62"/>
+    </row>
+    <row r="15" spans="1:13" ht="25">
+      <c r="A15" s="62" t="s">
         <v>60</v>
       </c>
-      <c r="B15" s="55"/>
-      <c r="C15" s="55"/>
-      <c r="D15" s="55"/>
-      <c r="E15" s="55" t="s">
+      <c r="B15" s="62"/>
+      <c r="C15" s="62"/>
+      <c r="D15" s="62"/>
+      <c r="E15" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="F15" s="55"/>
-      <c r="G15" s="55"/>
-      <c r="H15" s="56" t="s">
+      <c r="F15" s="62"/>
+      <c r="G15" s="62"/>
+      <c r="H15" s="59" t="s">
         <v>48</v>
       </c>
-      <c r="I15" s="57"/>
-      <c r="J15" s="58"/>
-      <c r="K15" s="56" t="s">
+      <c r="I15" s="60"/>
+      <c r="J15" s="61"/>
+      <c r="K15" s="59" t="s">
         <v>49</v>
       </c>
-      <c r="L15" s="57"/>
-      <c r="M15" s="58"/>
+      <c r="L15" s="60"/>
+      <c r="M15" s="61"/>
     </row>
     <row r="16" spans="1:13">
       <c r="A16" s="17"/>
@@ -21801,12 +21817,6 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="E3:G3"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="K3:M3"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="E15:G15"/>
     <mergeCell ref="H15:J15"/>
@@ -21822,6 +21832,12 @@
     <mergeCell ref="H11:J11"/>
     <mergeCell ref="K11:M11"/>
     <mergeCell ref="A14:M14"/>
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="K3:M3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -21830,91 +21846,91 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{675AB273-2180-584F-8A66-E764000A71E7}">
   <dimension ref="A1:L78"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.5"/>
   <cols>
-    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="30.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.77734375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="30.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.69140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.07421875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.765625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.69140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.07421875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.765625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="30.69140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.07421875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.765625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="30.69140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23.07421875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="25.5">
-      <c r="A1" s="69" t="s">
+    <row r="1" spans="1:12" ht="25">
+      <c r="A1" s="66" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
-      <c r="L1" s="69"/>
-    </row>
-    <row r="2" spans="1:12" s="6" customFormat="1" ht="59.1" customHeight="1">
-      <c r="A2" s="65" t="s">
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="66"/>
+      <c r="L1" s="66"/>
+    </row>
+    <row r="2" spans="1:12" s="6" customFormat="1" ht="59.15" customHeight="1">
+      <c r="A2" s="68" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="66"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="66"/>
-      <c r="G2" s="66"/>
-      <c r="H2" s="66"/>
-      <c r="I2" s="66"/>
-      <c r="J2" s="66"/>
-      <c r="K2" s="66"/>
-      <c r="L2" s="67"/>
-    </row>
-    <row r="3" spans="1:12" ht="25.5">
-      <c r="A3" s="55" t="s">
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="70"/>
+    </row>
+    <row r="3" spans="1:12" ht="25">
+      <c r="A3" s="62" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="55"/>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="55"/>
-      <c r="I3" s="55"/>
-      <c r="J3" s="55"/>
-      <c r="K3" s="55"/>
-      <c r="L3" s="55"/>
-    </row>
-    <row r="4" spans="1:12" ht="25.5">
-      <c r="A4" s="55" t="s">
+      <c r="B3" s="62"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
+      <c r="G3" s="62"/>
+      <c r="H3" s="62"/>
+      <c r="I3" s="62"/>
+      <c r="J3" s="62"/>
+      <c r="K3" s="62"/>
+      <c r="L3" s="62"/>
+    </row>
+    <row r="4" spans="1:12" ht="25">
+      <c r="A4" s="62" t="s">
         <v>60</v>
       </c>
-      <c r="B4" s="55"/>
-      <c r="C4" s="55"/>
-      <c r="D4" s="55" t="s">
+      <c r="B4" s="62"/>
+      <c r="C4" s="62"/>
+      <c r="D4" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="E4" s="55"/>
-      <c r="F4" s="55"/>
-      <c r="G4" s="55" t="s">
+      <c r="E4" s="62"/>
+      <c r="F4" s="62"/>
+      <c r="G4" s="62" t="s">
         <v>48</v>
       </c>
-      <c r="H4" s="55"/>
-      <c r="I4" s="55"/>
-      <c r="J4" s="55" t="s">
+      <c r="H4" s="62"/>
+      <c r="I4" s="62"/>
+      <c r="J4" s="62" t="s">
         <v>49</v>
       </c>
-      <c r="K4" s="55"/>
-      <c r="L4" s="55"/>
+      <c r="K4" s="62"/>
+      <c r="L4" s="62"/>
     </row>
     <row r="5" spans="1:12">
       <c r="A5" s="19" t="s">
@@ -22282,43 +22298,43 @@
       <c r="K21" s="25"/>
       <c r="L21" s="26"/>
     </row>
-    <row r="22" spans="1:12" ht="25.5">
-      <c r="A22" s="68" t="s">
+    <row r="22" spans="1:12" ht="25">
+      <c r="A22" s="67" t="s">
         <v>57</v>
       </c>
-      <c r="B22" s="68"/>
-      <c r="C22" s="68"/>
-      <c r="D22" s="68"/>
-      <c r="E22" s="68"/>
-      <c r="F22" s="68"/>
-      <c r="G22" s="68"/>
-      <c r="H22" s="68"/>
-      <c r="I22" s="68"/>
-      <c r="J22" s="68"/>
-      <c r="K22" s="68"/>
-      <c r="L22" s="68"/>
-    </row>
-    <row r="23" spans="1:12" ht="25.5">
-      <c r="A23" s="55" t="s">
+      <c r="B22" s="67"/>
+      <c r="C22" s="67"/>
+      <c r="D22" s="67"/>
+      <c r="E22" s="67"/>
+      <c r="F22" s="67"/>
+      <c r="G22" s="67"/>
+      <c r="H22" s="67"/>
+      <c r="I22" s="67"/>
+      <c r="J22" s="67"/>
+      <c r="K22" s="67"/>
+      <c r="L22" s="67"/>
+    </row>
+    <row r="23" spans="1:12" ht="25">
+      <c r="A23" s="62" t="s">
         <v>60</v>
       </c>
-      <c r="B23" s="55"/>
-      <c r="C23" s="55"/>
-      <c r="D23" s="55" t="s">
+      <c r="B23" s="62"/>
+      <c r="C23" s="62"/>
+      <c r="D23" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="E23" s="55"/>
-      <c r="F23" s="55"/>
-      <c r="G23" s="55" t="s">
+      <c r="E23" s="62"/>
+      <c r="F23" s="62"/>
+      <c r="G23" s="62" t="s">
         <v>48</v>
       </c>
-      <c r="H23" s="55"/>
-      <c r="I23" s="55"/>
-      <c r="J23" s="55" t="s">
+      <c r="H23" s="62"/>
+      <c r="I23" s="62"/>
+      <c r="J23" s="62" t="s">
         <v>49</v>
       </c>
-      <c r="K23" s="55"/>
-      <c r="L23" s="55"/>
+      <c r="K23" s="62"/>
+      <c r="L23" s="62"/>
     </row>
     <row r="24" spans="1:12">
       <c r="A24" s="19" t="s">
@@ -22686,43 +22702,43 @@
       <c r="K40" s="25"/>
       <c r="L40" s="26"/>
     </row>
-    <row r="41" spans="1:12" ht="25.5">
-      <c r="A41" s="68" t="s">
+    <row r="41" spans="1:12" ht="25">
+      <c r="A41" s="67" t="s">
         <v>58</v>
       </c>
-      <c r="B41" s="68"/>
-      <c r="C41" s="68"/>
-      <c r="D41" s="68"/>
-      <c r="E41" s="68"/>
-      <c r="F41" s="68"/>
-      <c r="G41" s="68"/>
-      <c r="H41" s="68"/>
-      <c r="I41" s="68"/>
-      <c r="J41" s="68"/>
-      <c r="K41" s="68"/>
-      <c r="L41" s="68"/>
-    </row>
-    <row r="42" spans="1:12" ht="25.5">
-      <c r="A42" s="55" t="s">
+      <c r="B41" s="67"/>
+      <c r="C41" s="67"/>
+      <c r="D41" s="67"/>
+      <c r="E41" s="67"/>
+      <c r="F41" s="67"/>
+      <c r="G41" s="67"/>
+      <c r="H41" s="67"/>
+      <c r="I41" s="67"/>
+      <c r="J41" s="67"/>
+      <c r="K41" s="67"/>
+      <c r="L41" s="67"/>
+    </row>
+    <row r="42" spans="1:12" ht="25">
+      <c r="A42" s="62" t="s">
         <v>60</v>
       </c>
-      <c r="B42" s="55"/>
-      <c r="C42" s="55"/>
-      <c r="D42" s="55" t="s">
+      <c r="B42" s="62"/>
+      <c r="C42" s="62"/>
+      <c r="D42" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="E42" s="55"/>
-      <c r="F42" s="55"/>
-      <c r="G42" s="55" t="s">
+      <c r="E42" s="62"/>
+      <c r="F42" s="62"/>
+      <c r="G42" s="62" t="s">
         <v>48</v>
       </c>
-      <c r="H42" s="55"/>
-      <c r="I42" s="55"/>
-      <c r="J42" s="55" t="s">
+      <c r="H42" s="62"/>
+      <c r="I42" s="62"/>
+      <c r="J42" s="62" t="s">
         <v>49</v>
       </c>
-      <c r="K42" s="55"/>
-      <c r="L42" s="55"/>
+      <c r="K42" s="62"/>
+      <c r="L42" s="62"/>
     </row>
     <row r="43" spans="1:12">
       <c r="A43" s="19" t="s">
@@ -23090,43 +23106,43 @@
       <c r="K59" s="25"/>
       <c r="L59" s="26"/>
     </row>
-    <row r="60" spans="1:12" ht="25.5">
-      <c r="A60" s="55" t="s">
+    <row r="60" spans="1:12" ht="25">
+      <c r="A60" s="62" t="s">
         <v>59</v>
       </c>
-      <c r="B60" s="55"/>
-      <c r="C60" s="55"/>
-      <c r="D60" s="55"/>
-      <c r="E60" s="55"/>
-      <c r="F60" s="55"/>
-      <c r="G60" s="55"/>
-      <c r="H60" s="55"/>
-      <c r="I60" s="55"/>
-      <c r="J60" s="55"/>
-      <c r="K60" s="55"/>
-      <c r="L60" s="55"/>
-    </row>
-    <row r="61" spans="1:12" ht="25.5">
-      <c r="A61" s="55" t="s">
+      <c r="B60" s="62"/>
+      <c r="C60" s="62"/>
+      <c r="D60" s="62"/>
+      <c r="E60" s="62"/>
+      <c r="F60" s="62"/>
+      <c r="G60" s="62"/>
+      <c r="H60" s="62"/>
+      <c r="I60" s="62"/>
+      <c r="J60" s="62"/>
+      <c r="K60" s="62"/>
+      <c r="L60" s="62"/>
+    </row>
+    <row r="61" spans="1:12" ht="25">
+      <c r="A61" s="62" t="s">
         <v>60</v>
       </c>
-      <c r="B61" s="55"/>
-      <c r="C61" s="55"/>
-      <c r="D61" s="55" t="s">
+      <c r="B61" s="62"/>
+      <c r="C61" s="62"/>
+      <c r="D61" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="E61" s="55"/>
-      <c r="F61" s="55"/>
-      <c r="G61" s="55" t="s">
+      <c r="E61" s="62"/>
+      <c r="F61" s="62"/>
+      <c r="G61" s="62" t="s">
         <v>48</v>
       </c>
-      <c r="H61" s="55"/>
-      <c r="I61" s="55"/>
-      <c r="J61" s="55" t="s">
+      <c r="H61" s="62"/>
+      <c r="I61" s="62"/>
+      <c r="J61" s="62" t="s">
         <v>49</v>
       </c>
-      <c r="K61" s="55"/>
-      <c r="L61" s="55"/>
+      <c r="K61" s="62"/>
+      <c r="L61" s="62"/>
     </row>
     <row r="62" spans="1:12">
       <c r="A62" s="19" t="s">
@@ -23496,13 +23512,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="G4:I4"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="A2:L2"/>
     <mergeCell ref="A61:C61"/>
     <mergeCell ref="D61:F61"/>
     <mergeCell ref="G61:I61"/>
@@ -23518,6 +23527,13 @@
     <mergeCell ref="G42:I42"/>
     <mergeCell ref="J42:L42"/>
     <mergeCell ref="A60:L60"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="G4:I4"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="A2:L2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -23526,79 +23542,79 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A7A1387-86E1-1C48-801D-0EFBC2B89D22}">
   <dimension ref="A1:M17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.5"/>
   <cols>
-    <col min="1" max="1" width="30.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.69140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.07421875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.765625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="25" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.07421875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.765625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="25" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.07421875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.765625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="25" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23.07421875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20.765625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="25.5">
-      <c r="A1" s="59" t="s">
+    <row r="1" spans="1:13" ht="25">
+      <c r="A1" s="56" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="60"/>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="70"/>
-    </row>
-    <row r="2" spans="1:13" ht="25.5">
-      <c r="A2" s="56" t="s">
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
+      <c r="H1" s="57"/>
+      <c r="I1" s="57"/>
+      <c r="J1" s="57"/>
+      <c r="K1" s="57"/>
+      <c r="L1" s="57"/>
+      <c r="M1" s="71"/>
+    </row>
+    <row r="2" spans="1:13" ht="25">
+      <c r="A2" s="59" t="s">
         <v>56</v>
       </c>
-      <c r="B2" s="57"/>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
-      <c r="E2" s="57"/>
-      <c r="F2" s="57"/>
-      <c r="G2" s="57"/>
-      <c r="H2" s="57"/>
-      <c r="I2" s="57"/>
-      <c r="J2" s="57"/>
-      <c r="K2" s="57"/>
-      <c r="L2" s="57"/>
-      <c r="M2" s="58"/>
-    </row>
-    <row r="3" spans="1:13" s="6" customFormat="1" ht="25.5">
-      <c r="A3" s="55" t="s">
+      <c r="B2" s="60"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
+      <c r="H2" s="60"/>
+      <c r="I2" s="60"/>
+      <c r="J2" s="60"/>
+      <c r="K2" s="60"/>
+      <c r="L2" s="60"/>
+      <c r="M2" s="61"/>
+    </row>
+    <row r="3" spans="1:13" s="6" customFormat="1" ht="25">
+      <c r="A3" s="62" t="s">
         <v>60</v>
       </c>
-      <c r="B3" s="55"/>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55" t="s">
+      <c r="B3" s="62"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="F3" s="55"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="56" t="s">
+      <c r="F3" s="62"/>
+      <c r="G3" s="62"/>
+      <c r="H3" s="59" t="s">
         <v>48</v>
       </c>
-      <c r="I3" s="57"/>
-      <c r="J3" s="58"/>
-      <c r="K3" s="56" t="s">
+      <c r="I3" s="60"/>
+      <c r="J3" s="61"/>
+      <c r="K3" s="59" t="s">
         <v>49</v>
       </c>
-      <c r="L3" s="57"/>
-      <c r="M3" s="58"/>
+      <c r="L3" s="60"/>
+      <c r="M3" s="61"/>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="38"/>
@@ -23656,45 +23672,45 @@
       <c r="L5" s="39"/>
       <c r="M5" s="39"/>
     </row>
-    <row r="6" spans="1:13" ht="25.5">
-      <c r="A6" s="56" t="s">
+    <row r="6" spans="1:13" ht="25">
+      <c r="A6" s="59" t="s">
         <v>57</v>
       </c>
-      <c r="B6" s="57"/>
-      <c r="C6" s="57"/>
-      <c r="D6" s="57"/>
-      <c r="E6" s="57"/>
-      <c r="F6" s="57"/>
-      <c r="G6" s="57"/>
-      <c r="H6" s="57"/>
-      <c r="I6" s="57"/>
-      <c r="J6" s="57"/>
-      <c r="K6" s="57"/>
-      <c r="L6" s="57"/>
-      <c r="M6" s="58"/>
-    </row>
-    <row r="7" spans="1:13" s="6" customFormat="1" ht="25.5">
-      <c r="A7" s="55" t="s">
+      <c r="B6" s="60"/>
+      <c r="C6" s="60"/>
+      <c r="D6" s="60"/>
+      <c r="E6" s="60"/>
+      <c r="F6" s="60"/>
+      <c r="G6" s="60"/>
+      <c r="H6" s="60"/>
+      <c r="I6" s="60"/>
+      <c r="J6" s="60"/>
+      <c r="K6" s="60"/>
+      <c r="L6" s="60"/>
+      <c r="M6" s="61"/>
+    </row>
+    <row r="7" spans="1:13" s="6" customFormat="1" ht="25">
+      <c r="A7" s="62" t="s">
         <v>60</v>
       </c>
-      <c r="B7" s="55"/>
-      <c r="C7" s="55"/>
-      <c r="D7" s="55"/>
-      <c r="E7" s="55" t="s">
+      <c r="B7" s="62"/>
+      <c r="C7" s="62"/>
+      <c r="D7" s="62"/>
+      <c r="E7" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="F7" s="55"/>
-      <c r="G7" s="55"/>
-      <c r="H7" s="56" t="s">
+      <c r="F7" s="62"/>
+      <c r="G7" s="62"/>
+      <c r="H7" s="59" t="s">
         <v>48</v>
       </c>
-      <c r="I7" s="57"/>
-      <c r="J7" s="58"/>
-      <c r="K7" s="56" t="s">
+      <c r="I7" s="60"/>
+      <c r="J7" s="61"/>
+      <c r="K7" s="59" t="s">
         <v>49</v>
       </c>
-      <c r="L7" s="57"/>
-      <c r="M7" s="58"/>
+      <c r="L7" s="60"/>
+      <c r="M7" s="61"/>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="38"/>
@@ -23752,45 +23768,45 @@
       <c r="L9" s="25"/>
       <c r="M9" s="25"/>
     </row>
-    <row r="10" spans="1:13" ht="25.5">
-      <c r="A10" s="56" t="s">
+    <row r="10" spans="1:13" ht="25">
+      <c r="A10" s="59" t="s">
         <v>58</v>
       </c>
-      <c r="B10" s="57"/>
-      <c r="C10" s="57"/>
-      <c r="D10" s="57"/>
-      <c r="E10" s="57"/>
-      <c r="F10" s="57"/>
-      <c r="G10" s="57"/>
-      <c r="H10" s="57"/>
-      <c r="I10" s="57"/>
-      <c r="J10" s="57"/>
-      <c r="K10" s="57"/>
-      <c r="L10" s="57"/>
-      <c r="M10" s="58"/>
-    </row>
-    <row r="11" spans="1:13" s="6" customFormat="1" ht="25.5">
-      <c r="A11" s="55" t="s">
+      <c r="B10" s="60"/>
+      <c r="C10" s="60"/>
+      <c r="D10" s="60"/>
+      <c r="E10" s="60"/>
+      <c r="F10" s="60"/>
+      <c r="G10" s="60"/>
+      <c r="H10" s="60"/>
+      <c r="I10" s="60"/>
+      <c r="J10" s="60"/>
+      <c r="K10" s="60"/>
+      <c r="L10" s="60"/>
+      <c r="M10" s="61"/>
+    </row>
+    <row r="11" spans="1:13" s="6" customFormat="1" ht="25">
+      <c r="A11" s="62" t="s">
         <v>60</v>
       </c>
-      <c r="B11" s="55"/>
-      <c r="C11" s="55"/>
-      <c r="D11" s="55"/>
-      <c r="E11" s="55" t="s">
+      <c r="B11" s="62"/>
+      <c r="C11" s="62"/>
+      <c r="D11" s="62"/>
+      <c r="E11" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="55"/>
-      <c r="G11" s="55"/>
-      <c r="H11" s="56" t="s">
+      <c r="F11" s="62"/>
+      <c r="G11" s="62"/>
+      <c r="H11" s="59" t="s">
         <v>48</v>
       </c>
-      <c r="I11" s="57"/>
-      <c r="J11" s="58"/>
-      <c r="K11" s="56" t="s">
+      <c r="I11" s="60"/>
+      <c r="J11" s="61"/>
+      <c r="K11" s="59" t="s">
         <v>49</v>
       </c>
-      <c r="L11" s="57"/>
-      <c r="M11" s="58"/>
+      <c r="L11" s="60"/>
+      <c r="M11" s="61"/>
     </row>
     <row r="12" spans="1:13">
       <c r="A12" s="38"/>
@@ -23848,45 +23864,45 @@
       <c r="L13" s="41"/>
       <c r="M13" s="41"/>
     </row>
-    <row r="14" spans="1:13" ht="25.5">
-      <c r="A14" s="56" t="s">
+    <row r="14" spans="1:13" ht="25">
+      <c r="A14" s="59" t="s">
         <v>59</v>
       </c>
-      <c r="B14" s="57"/>
-      <c r="C14" s="57"/>
-      <c r="D14" s="57"/>
-      <c r="E14" s="57"/>
-      <c r="F14" s="57"/>
-      <c r="G14" s="57"/>
-      <c r="H14" s="57"/>
-      <c r="I14" s="57"/>
-      <c r="J14" s="57"/>
-      <c r="K14" s="57"/>
-      <c r="L14" s="57"/>
-      <c r="M14" s="58"/>
-    </row>
-    <row r="15" spans="1:13" s="6" customFormat="1" ht="25.5">
-      <c r="A15" s="55" t="s">
+      <c r="B14" s="60"/>
+      <c r="C14" s="60"/>
+      <c r="D14" s="60"/>
+      <c r="E14" s="60"/>
+      <c r="F14" s="60"/>
+      <c r="G14" s="60"/>
+      <c r="H14" s="60"/>
+      <c r="I14" s="60"/>
+      <c r="J14" s="60"/>
+      <c r="K14" s="60"/>
+      <c r="L14" s="60"/>
+      <c r="M14" s="61"/>
+    </row>
+    <row r="15" spans="1:13" s="6" customFormat="1" ht="25">
+      <c r="A15" s="62" t="s">
         <v>60</v>
       </c>
-      <c r="B15" s="55"/>
-      <c r="C15" s="55"/>
-      <c r="D15" s="55"/>
-      <c r="E15" s="55" t="s">
+      <c r="B15" s="62"/>
+      <c r="C15" s="62"/>
+      <c r="D15" s="62"/>
+      <c r="E15" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="F15" s="55"/>
-      <c r="G15" s="55"/>
-      <c r="H15" s="56" t="s">
+      <c r="F15" s="62"/>
+      <c r="G15" s="62"/>
+      <c r="H15" s="59" t="s">
         <v>48</v>
       </c>
-      <c r="I15" s="57"/>
-      <c r="J15" s="58"/>
-      <c r="K15" s="56" t="s">
+      <c r="I15" s="60"/>
+      <c r="J15" s="61"/>
+      <c r="K15" s="59" t="s">
         <v>49</v>
       </c>
-      <c r="L15" s="57"/>
-      <c r="M15" s="58"/>
+      <c r="L15" s="60"/>
+      <c r="M15" s="61"/>
     </row>
     <row r="16" spans="1:13">
       <c r="A16" s="38"/>
@@ -23946,12 +23962,6 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="E3:G3"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="K3:M3"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="E15:G15"/>
     <mergeCell ref="H15:J15"/>
@@ -23967,6 +23977,12 @@
     <mergeCell ref="H11:J11"/>
     <mergeCell ref="K11:M11"/>
     <mergeCell ref="A14:M14"/>
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="K3:M3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>